<commit_message>
niente owl:sameAs per i giudizi d'identità; chora:housedIn per istituzione e sede (T-31, D-044)
Castello <-> Castel Gandolfo: asserzione d'identificazione di Lorenzo,
non adottata (DC-04). Santo Stefano del Cacco e Regina Coeli: housedIn
Collegio Romano e via della Lungara. L'ETL rifiuta id interni in sameAs.
Aggiornati build_geojson.py, D-009, D-011. ABox 24.575 -> 24.588,
full 25.901 -> 25.921, SHACL conforme.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Assertions.xlsx
+++ b/data/source/xlsx/Assertions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,6 +480,58 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>A-0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>identification</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>narrativeplace/castello</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_castel_gandolfo</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>annotator/lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>annotator/lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Lettura del censimento: la «stazione di Castello» (QP 279) come Castel Gandolfo, lettura immediata del toponimo. Identificazione contesa (DC-04): Manzotti 2010, p. 293 legge Castel Savello; la sua lettura entra in fase 3. Non adottata finché DC-04 non è deciso.</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Sostituisce owl:sameAs gaz_castello &lt;-&gt; gaz_castel_gandolfo (D-044)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
incertezza tipizzata: tipo, asse, origine, autore; 8 casi documentati (T-34, D-047)
Tre schemi SKOS (tipo con i sottotipi della discrepanza, asse, origine);
assenza = non analizzato. Casi: Casal Bruciato, Castello, Simonetti,
Robine, edicola, Ernici/Simbruini, Càrsoli, Direttissima, in bozza.
confidence e hasFuzzinessLevel invariati. TBox 827 -> 971,
ABox 25.579 -> 25.755, SHACL conforme.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Assertions.xlsx
+++ b/data/source/xlsx/Assertions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O54"/>
+  <dimension ref="A1:Q62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,6 +492,16 @@
           <t>Review_Status</t>
         </is>
       </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Uncertainty_Axis</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Uncertainty_Origin</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3804,6 +3814,608 @@
       <c r="O54" t="inlineStr">
         <is>
           <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>U-0001</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>uncertainty</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>narrativeplace/casal_bruciato</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>chora:Confusion</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>agent/manzotti</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>annotator/lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Manzotti 2010</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>268–269</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>La topografia di Gadda «pare combinare e forse confondere» le due ferrovie, «fondandosi […] più sulla memoria di escursioni in loco, che sui rilievi delle carte»; TCI e testo tra le due ferrovie, IGM a ovest della Roma–Napoli. Discrepanza fra testo e repertorio, non corretta (D-037).</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>Bozza T-34 (D-047): classificazione da validare in REVIEW_2</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>geometria</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>documentaria</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>U-0002</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>uncertainty</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>narrativeplace/castello</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>chora:ContestedIdentification</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>annotator/lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>annotator/lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Manzotti 2010</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>293</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Due identificazioni concorrenti della «stazione di Castello» (QP 279): Castel Gandolfo (lettura immediata, A-0001) e Castel Savello (Manzotti, A-0002, adottata). Cap. 4, § 4.4 (r. 107).</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>Bozza T-34 (D-047): classificazione da validare in REVIEW_2</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>identificazione</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>costruttiva</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>U-0003</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>uncertainty</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>narrativeplace/palazzo_simonetti</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>chora:ContestedIdentification</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>annotator/lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>annotator/lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Pinotti 2025</t>
+        </is>
+      </c>
+      <c r="H57" t="n">
+        <v>78</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Quale palazzo reale sta dietro il «palazzo Simonetti» in via Lanza (QP 177): il palazzo Simonetti / De Carolis in via Lata del dattiloscritto (Pinotti) o il palazzo Odescalchi Simonetti di via Vittoria Colonna (Terzoli, cit. ivi). Cap. 4, § 4.2 (r. 45).</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>Bozza T-34 (D-047): classificazione da validare in REVIEW_2</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>identificazione</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>documentaria</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>U-0004</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>uncertainty</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>narrativeplace/robine_vecchie</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>chora:Discrepancy</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>annotator/lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>annotator/lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Terzoli 2015</t>
+        </is>
+      </c>
+      <c r="H58" t="n">
+        <v>491</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>«Robine Vecchie» (QP 169) non è registrato nelle carte topografiche: refuso per «Robinie vecchie» o «Rovine vecchie», oppure «ironico abbassamento» delle Rovine della zona; Pinotti conserva la lezione. Cap. 4, § 4.3 (r. 83).</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>Bozza T-34 (D-047): classificazione da validare in REVIEW_2</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>documentaria</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>U-0005</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>uncertainty</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>narrativeplace/edicola_due_santi</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>chora:Incompleteness</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>annotator/lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>annotator/lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Manzotti 2010</t>
+        </is>
+      </c>
+      <c r="H59" t="n">
+        <v>246</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Il tabernacolo ha traccia nella piantina dei Castelli del Touring (Manzotti), ma il progetto non dispone di una coordinata: la posizione deriva da Due Santi con uno scarto dichiarato di circa 40 m (D-031); il volume TCI citato è da verificare (DC-03).</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>Bozza T-34 (D-047): classificazione da validare in REVIEW_2</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>geometria</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>costruttiva</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>U-0006</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>uncertainty</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>narrativeplace/monti_ernici</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>chora:NonSpecificity</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>agent/manzotti</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>annotator/lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Manzotti 2010</t>
+        </is>
+      </c>
+      <c r="H60" t="n">
+        <v>290</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>«d'in vetta al crinale degli Ernici o dei Simbruini» (QP 215): identificazione per disgiunzione, non risolta dal testo (WO T-16; Cap. 4, § 4.4).</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>Bozza T-34 (D-047): classificazione da validare in REVIEW_2</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>identificazione</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>documentaria</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>U-0007</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>uncertainty</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>narrativeplace/carsoli</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>chora:Oversight</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>agent/manzotti</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>annotator/lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Manzotti 2010</t>
+        </is>
+      </c>
+      <c r="H61" t="n">
+        <v>254</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>«Càrsoli» (QP 210) in luogo della grafia corretta Carsòli, «frutto verosimilmente di un'attrazione analogica con la vicina Àrsoli» (Cap. 4, § 4.4, r. 111). Discrepanza di forma registrata, non corretta.</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>Bozza T-34 (D-047): classificazione da validare in REVIEW_2</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>documentaria</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>U-0008</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>uncertainty</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>narrativeplace/direttissima_roma_napoli</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>chora:Anachronism</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>agent/manzotti</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>annotator/lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Manzotti 2010</t>
+        </is>
+      </c>
+      <c r="H62" t="n">
+        <v>270</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>La direttissima Roma–Napoli fu ultimata e inaugurata dopo gli eventi narrati (marzo 1927) (Cap. 4, § 4.4, r. 111). Anacronismo registrato, non corretto.</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>Bozza T-34 (D-047): classificazione da validare in REVIEW_2</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>identificazione</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>documentaria</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
partizione Roma città / campagna romana come ipotesi attribuita (T-37, D-050)
Partition e PartitionZone; la partizione è soggetto di un'asserzione
(P-0001, Lorenzo, adottata, bozza). Criterio: distanza dell'ancora primaria
dal Campidoglio (città entro 10 km, campagna fra 10 e 30). 221 luoghi
assegnati (162 + 59), 33 casi di confine in revisione. Shape 12, IQ15.
TBox 1.049 -> 1.069, ABox 25.917 -> 26.169, SHACL conforme.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Assertions.xlsx
+++ b/data/source/xlsx/Assertions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q68"/>
+  <dimension ref="A1:Q69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4847,6 +4847,78 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>P-0001</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>partition</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>partition/citta_campagna</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>zone/roma_citta|zone/campagna_romana</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Capitolo 4</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>§ 4.1, § 4.6 (R20)</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>Partizione Roma città / campagna romana, lettura adottata dal progetto. Criterio: distanza dell'ancora primaria del luogo dal Campidoglio; città fino a 10 km (nei dati il primo luogo di campagna, Castel di Leva, è a 12,9 km; l'ultimo urbano, l'Acqua Marcia, a 8,4), campagna fra 10 e 30 km. Non si assegnano d'ufficio entità lineari o areali che attraversano la soglia, luoghi Imagined, luoghi senza ancora, il litorale e la fascia fra 30 e 60 km: sono i casi di confine (REVIEW_2).</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>Il poligono comunale di roma.geojson è scartato come criterio: include l'Agro romano (Divino Amore, Castel di Leva, Tor di Gheppio) ed esclude il Vaticano. Altre letture della partizione (Roggia, Perosa, Savettieri, Alfano, Calvino): fase 3.</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
storia delle revisioni: tre letture del censimento superate (T-38, D-051)
prov:wasRevisionOf per edicola ai Due Santi (Invented, ex Imagined del
censimento -> Imported), Casal Bruciato (Tiburtino -> casale dell'Agro,
nuova identificazione adottata) e palazzo Simonetti (Imported ->
Transformed). La permutazione è una historyNote dello schema. Shape 13, IQ16.
TBox 1.069 -> 1.070, ABox 26.169 -> 26.249, SHACL conforme.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Assertions.xlsx
+++ b/data/source/xlsx/Assertions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q69"/>
+  <dimension ref="A1:Q73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1793,6 +1793,11 @@
           <t>Cap. 4, n. 24 (r. 601): «L'edicola dei Due Santi (QP 216, 219), che una prima lettura direbbe inventata, conserva secondo Manzotti una traccia nella piantina dei Castelli della guida del Touring». Imported (D-031); revisione della lettura di censimento (Imagined) in T-38.</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>C-edicola_due_santi</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>2026-10-09</t>
@@ -2416,6 +2421,11 @@
           <t>Palazzo reale (Simonetti o De Carolis) in via Lata, che QP 177 colloca in via Lanza, dove non esiste: trasformazione per rilocazione (D-036). Cap. 4, § 4.2 (r. 45): «la stampa del 1957 colloca in via Lanza – abbinamento privo di riscontro reale per l'edificio […] –, laddove il dattiloscritto registrava correttamente via Lata».</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>C-palazzo_simonetti</t>
+        </is>
+      </c>
       <c r="L32" t="inlineStr">
         <is>
           <t>2026-10-09</t>
@@ -4916,6 +4926,264 @@
       <c r="O69" t="inlineStr">
         <is>
           <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>C-edicola_due_santi</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>narrativeplace/edicola_due_santi</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>chora:Invented</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Censimento GaddAtlas</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>Lettura del censimento: «Edicola immaginata», parte dell'orto/vigna dei Due Santi, senza ancoraggio. Nel censimento l'etichetta era «Imagined», che prima della correzione dello schema (D-030) designava il luogo fittizio in una geografia nota, oggi Invented.</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>Superata da S-edicola_due_santi (Manzotti 2010, p. 246; D-031).</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>C-palazzo_simonetti</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>narrativeplace/palazzo_simonetti</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>chora:Imported</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Censimento GaddAtlas</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Lettura del censimento: palazzo reale, ancorato a via Lanza dove lo pone QP 177.</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>Superata da S-palazzo_simonetti (Pinotti 2025, p. 78; D-036): in via Lanza non esiste un palazzo Simonetti.</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>C-casal_bruciato</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>identification</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>narrativeplace/casal_bruciato</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_casal_bruciato</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Censimento GaddAtlas</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Lettura del censimento: Casal Bruciato identificato con il quartiere omonimo del Tiburtino (41,9070 N 12,5506 E).</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>L'entità gaz_casal_bruciato è stata eliminata (D-029): l'IRI resta come valore di questa lettura superata. Passaggio intermedio D-029 (luogo trasformato senza referente, ancorato a Marino, Albano, Pavona e Santa Palomba), superato da D-037.</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>I-casal_bruciato</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>identification</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>narrativeplace/casal_bruciato</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_casale_abbruciato</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Manzotti 2010</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>268–269; Tavv. VI–VII, pp. 300–301</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Casal Bruciato è il casale dell'Agro romano a sud di Roma, «Casal(e) Bruciato / Abbruciato / Abbrusciato» (Nibby, Dintorni di Roma, p. 569), fra le ferrovie Roma–Napoli e Roma–Velletri; posizione adottata TCI (D-037).</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>C-casal_bruciato</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>validata</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
percorsi tipizzati: sei tipi, ventuno percorsi (T-54, D-060)
RouteTypeScheme (compiuto, indicato, sognato, inferito, direzionale,
proposto) assegnato da asserzioni attribuite (R-0001..R-0021, bozza);
hasRouteType derivato dalla lettura adottata, routeType nel GeoJSON.
Separato il percorso di QP 169 da quello di QP 297; nuovi percorsi QP 212
(sognato) e QP 237 (indicato). Shape 19.
TBox 1.230 -> 1.306, ABox 27.336 -> 27.854, percorsi 18 -> 21.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Assertions.xlsx
+++ b/data/source/xlsx/Assertions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q77"/>
+  <dimension ref="A1:Q98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5451,6 +5451,1455 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>R-0001</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>route/tragitto_torraccio_ponte_divino_amore</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>chora:CompletedRoute</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>QP</t>
+        </is>
+      </c>
+      <c r="H78" t="n">
+        <v>297</v>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>«Discesero ai Torraccio […] Svoltarono sull'Appia a li Due Santi […] Valicò invece il binario»: Ingravallo, Di Pietrantonio, l'autista e Runzato percorrono il tragitto in auto.</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>L'ultimo nodo (ponte del Divino Amore) è un termine di paragone («simile a quello ch'era due chilometri più a nord, presso il ponte»), non un punto attraversato: da rivedere.</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>R-0002</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>route/tragitto_santarella_torraccio_divino_amore</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>chora:InferredRoute</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>QP</t>
+        </is>
+      </c>
+      <c r="H79" t="n">
+        <v>169</v>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>La motocicletta di Santarella «si preannunciava di lontano, dal Torraccio, […] o dal Divino Amore»: le provenienze si ricavano dal rumore, «altre volte» da un luogo o dall'altro.</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>Separato dal tragitto di QP 297 (D-060). È un elenco disgiuntivo e abituale di provenienze, non una sequenza: potrebbe non essere un percorso.</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>R-0003</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>route/tragitto_tenenza_due_santi</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>chora:CompletedRoute</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>QP</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>208–215</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Pestalozzi e Cocullo scendono dalla caserma di Marino alla porta del borgo, prendono l'Appia, passano la Fontana e si fermano ai Due Santi.</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>R-0004</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>route/tragitto_brancaccio_piazza_san_giovanni</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>chora:CompletedRoute</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>QP</t>
+        </is>
+      </c>
+      <c r="H81" t="n">
+        <v>292</v>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>«A largo Brancaccio, mentre che staveno svortando in via Merulana verso piazza San Giovanni»: il tragitto è in corso.</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>L'ultimo nodo è una direzione («verso piazza San Giovanni»): l'arrivo non è narrato.</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>R-0005</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>route/tragitto_viminale_merulana</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>chora:CompletedRoute</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>QP</t>
+        </is>
+      </c>
+      <c r="H82" t="n">
+        <v>25</v>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>«Saliti sul PV e discesi appunto al Viminale, presero il tram di San Giovanni […] raggiunsero il civico ducentodicinnove».</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>R-0006</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>route/tragitto_appia_falcognana</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>chora:IndicatedRoute</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>QP</t>
+        </is>
+      </c>
+      <c r="H83" t="n">
+        <v>238</v>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>«La strada era una sola, pe fortuna, salvo il primo pezzo però: la statale, l'Appia, poi ad angolo retto la deviazione della provinciale, pe Falcognana»: la strada spiegata dopo le indicazioni di Camilla (QP 237).</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>Incerto fra indicato e compiuto: il passo descrive la strada, il viaggio segue.</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>R-0007</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>route/tragitto_agostino_aquiro</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>chora:CompletedRoute</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>QP</t>
+        </is>
+      </c>
+      <c r="H84" t="n">
+        <v>40</v>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Il commendator Angeloni e i suoi pari «sogliono deambulare» da Sant'Agostino a Santa Maria in Aquiro.</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>Percorso abituale (iterativo).</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>R-0008</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>route/tragitto_cecchina_anziate</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>chora:CompletedRoute</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>QP</t>
+        </is>
+      </c>
+      <c r="H85" t="n">
+        <v>173</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>La motocicletta di Santarella «infilava […] la mala curva d'aa stazione d'aa Cecchina», poi si fermava a Santa Palomba e a Campoleone, «il caso richiedendo».</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>Percorso abituale (iterativo), con fermate eventuali.</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>R-0009</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>route/tragitto_colonna_treccani</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>chora:CompletedRoute</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>QP</t>
+        </is>
+      </c>
+      <c r="H86" t="n">
+        <v>40</v>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Angeloni e i suoi pari «si avventurano» per via Colonna, piazza de Pietra, via de Pietra fino al Corso.</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>Percorso abituale (iterativo).</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>R-0010</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>route/tragitto_frattocchie_ciampino</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>chora:InferredRoute</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>QP</t>
+        </is>
+      </c>
+      <c r="H87" t="n">
+        <v>174</v>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>«Oppure a metà le Frattocchie, doveva spengere: al passaggio dell'Appia, o a Ca' Francesi, a Tor Ser Paolo, alla stazione di Ciampino»: luoghi alternativi della fermata.</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>Come QP 169: elenco disgiuntivo e abituale, non una sequenza.</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>R-0011</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>route/tragitto_monti_piazza_esedra</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>chora:CompletedRoute</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>QP</t>
+        </is>
+      </c>
+      <c r="H88" t="n">
+        <v>182</v>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Diomede «si differiva passo passo da un quartiere all'altro: monticiano a le dieci, trasteverino a le quattro, a Piazza Colonna o a l'Esedra».</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>Percorso abituale (iterativo); l'ultimo nodo è disgiuntivo («o»).</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>R-0012</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>route/tragitto_rocca_di_papa_monte_nuncupale</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>chora:CompletedRoute</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>QP</t>
+        </is>
+      </c>
+      <c r="H89" t="n">
+        <v>173</v>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Santarella «da Rocca di Papa a Castel Savelli, giù: da Rocca Orsina al Monte Nuncupale, su».</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>Percorso abituale (iterativo).</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>R-0013</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>route/tragitto_chiara_pantheon</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>chora:CompletedRoute</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>QP</t>
+        </is>
+      </c>
+      <c r="H90" t="n">
+        <v>41</v>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Di quaresima Angeloni e i suoi pari «si contentano lungheggiar Santa Chiara […] imboccheno la Palommella e sfioreno er dedietro ar Panteone».</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>Percorso abituale (iterativo).</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>R-0014</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>route/tragitto_duesanti_frattocchie</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>chora:CompletedRoute</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>QP</t>
+        </is>
+      </c>
+      <c r="H91" t="n">
+        <v>56</v>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>La corsa del tram dei Castelli: «Ai Due Santi, al Torraccio, a le Frattocchie […] era salita una quantità di persone».</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>R-0015</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>route/tragitto_policlinico_san_lorenzo_al_verano</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>chora:CompletedRoute</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>QP</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>139–140</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Il corteo funebre «spostò dar Policlinico a le otto […] tajarono pe la direttissima der viale Regina Margherita […] arrivarono a San Lorenzo ar Verano».</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>R-0016</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>route/tragitto_marino_albano_laziale</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>chora:DirectionalRoute</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>QP</t>
+        </is>
+      </c>
+      <c r="H93" t="n">
+        <v>278</v>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Santarella «era a percorrere sulla sua motocicletta la via provinciale da Marino ad Albano»: il passo dà la strada e la sua direzione, non il tratto percorso.</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>Alternativa: compiuto. Il Cap. 4 (r. 194) chiama questo tipo «presunto».</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>R-0017</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>route/tragitto_marino_due_santi</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>chora:CompletedRoute</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>QP</t>
+        </is>
+      </c>
+      <c r="H94" t="n">
+        <v>206</v>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Pestalozzi «usciva (in motocicletta) dalla caserma […] di Marino per catapultarsi alla bottega-laboratorio».</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>R-0018</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>route/tragitto_marino_santo_stefano</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>chora:CompletedRoute</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>QP</t>
+        </is>
+      </c>
+      <c r="H95" t="n">
+        <v>153</v>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>«arrivò a Santo Stefano in motocicletta il brigadiere Pestalozzi […] latore di un rapporto […] della Tenenza».</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>La partenza dalla Tenenza è inferita dal rapporto. L'ordine dei nodi è invertito (1 Santo Stefano, 2 Tenenza): da correggere.</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>R-0019</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>route/tragitto_merulana_policlinico</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>chora:CompletedRoute</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>QP</t>
+        </is>
+      </c>
+      <c r="H96" t="n">
+        <v>93</v>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>L'autorità giudiziaria «era intervenuta […] a via Merulana, indi al Policlinico».</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>Il focalizzatore registrato è Liliana, ma chi si sposta è il giudice istruttore; se il percorso è quello del corpo, è un oggetto (DM-03, escluso).</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>R-0020</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>route/tragitto_sogno_casal_bruciato_campo_morto</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>chora:DreamedRoute</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>QP</t>
+        </is>
+      </c>
+      <c r="H97" t="n">
+        <v>212</v>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Il sogno di Pestalozzi: «al passaggio a livello di Casal Bruciato il vetrone girasole... per fil a dest!», il Roma-Napoli che «filava filava», la fuga «verso le gore senza foce del Campo Morto».</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>Nuovo percorso (D-060). La lettura di Manzotti di «per fil a dest» (2010, p. 269) è una nota attribuita di fase 3.</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>R-0021</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>route/tragitto_castel_di_leva_casal_bruciato</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>chora:IndicatedRoute</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>QP</t>
+        </is>
+      </c>
+      <c r="H98" t="n">
+        <v>237</v>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Camilla indica la strada: «Pe la strada de Castel de Leva, fino ar ponte: poi, a sinistra, fino ar passaggio a livello de Casal Bruciato».</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>Nuovo percorso (D-060). Il nodo finale è il passaggio a livello: nei dati l'occorrenza è di casal_bruciato.</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
statuti dopo REVIEW_2: castello Imported, nuova definizione di Imagined (D-061)
Riassegnazioni a Invented respinte: i cinque Imagined restano tali.
castello -> Imported sull'identificazione adottata (Manzotti 2010, p. 293).
Definizione di Imagined di Lorenzo in TBox, CLAUDE.md, DATA_CHECKS.
Statuti 261/30/13/5; avvertenze SHACL 52 -> 51.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Assertions.xlsx
+++ b/data/source/xlsx/Assertions.xlsx
@@ -1459,7 +1459,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>chora:Invented</t>
+          <t>chora:Imported</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1487,7 +1487,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Luogo testuale della «stazione di Castello» (QP 279), bersaglio di due identificazioni concorrenti (Cap. 4, § 4.3, r. 93; § 4.4, r. 107): Castel Gandolfo (LS, A-0001) e Castel Savello (Manzotti 2010, p. 293, A-0002, adottata). Statuto da rivedere alla luce della lettura adottata (REVIEW_2).</t>
+          <t>La «stazione di Castello» (QP 279) è la stazione dei carabinieri di Castel Savello: identificazione adottata A-0002 (Manzotti 2010, p. 293). Il luogo testuale nomina in forma ellittica un luogo reale: statuto Imported. La lettura alternativa (Castel Gandolfo, A-0001) è anch'essa un luogo reale.</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1497,17 +1497,17 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Decisione di LS (9/10/2026, REVIEW_2 § 2); prima Invented (bozza T-33).</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>lettura critica</t>
+          <t>prova referenziale</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
percorsi dopo REVIEW_2: QP 297, 153, 93 invariati nei dati (D-064)
Ordine dei nodi di QP 153 già quello del testo; focalizzatrice di QP 93
Liliana; Mappamonno già con Mussolini. Aggiornate le note di R-0001,
R-0018, R-0019. Triple invariate.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Assertions.xlsx
+++ b/data/source/xlsx/Assertions.xlsx
@@ -5507,7 +5507,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>L'ultimo nodo (ponte del Divino Amore) è un termine di paragone («simile a quello ch'era due chilometri più a nord, presso il ponte»), non un punto attraversato: da rivedere.</t>
+          <t>L'ultimo nodo (ponte del Divino Amore) è un termine di paragone («simile a quello ch'era due chilometri più a nord, presso il ponte»): lasciato invariato per decisione di LS (9/10/2026, D-064).</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -6676,7 +6676,7 @@
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>La partenza dalla Tenenza è inferita dal rapporto. L'ordine dei nodi è invertito (1 Santo Stefano, 2 Tenenza): da correggere.</t>
+          <t>Nodi nell'ordine di occorrenza nel testo (decisione di LS, 9/10/2026, D-064): Santo Stefano 1, Tenenza 2. La partenza dalla Tenenza è inferita dal rapporto.</t>
         </is>
       </c>
       <c r="N95" t="inlineStr">
@@ -6746,7 +6746,7 @@
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>Il focalizzatore registrato è Liliana, ma chi si sposta è il giudice istruttore; se il percorso è quello del corpo, è un oggetto (DM-03, escluso).</t>
+          <t>Focalizzatrice del tragitto: Liliana, come nel database (decisione di LS, 9/10/2026, D-064).</t>
         </is>
       </c>
       <c r="N96" t="inlineStr">

</xml_diff>

<commit_message>
pattern HiCO: la lettura generata dall'atto interpretativo (B1, D-067)
Assertion e SpatialInterpretation generate da hico:InterpretationAct (tipo,
criterio, fonte, pagina, motivazione, associazioni); codifica distinta
(EncodingActivity, wasInformedBy) quando l'autore è uno studioso, con la
data della fonte sull'atto. Sources.tsv (8 fonti). reifiesProperty;
identifiedWith materializzata. HiCO dichiarato in locale.
TBox 1.320 -> 1.422, ABox 27.857 -> 32.385, SHACL conforme (48).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Assertions.xlsx
+++ b/data/source/xlsx/Assertions.xlsx
@@ -534,6 +534,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>no</t>
@@ -598,7 +603,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Manzotti 2010</t>
+          <t>manzotti_2010</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -666,6 +671,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>si</t>
@@ -728,6 +738,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>si</t>
@@ -961,6 +976,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
           <t>si</t>
@@ -1023,6 +1043,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
           <t>si</t>
@@ -1085,6 +1110,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
           <t>si</t>
@@ -1147,6 +1177,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
           <t>si</t>
@@ -1211,7 +1246,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Manzotti 2010</t>
+          <t>manzotti_2010</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1281,6 +1316,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
           <t>si</t>
@@ -1402,7 +1442,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Manzotti 2010</t>
+          <t>manzotti_2010</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1474,7 +1514,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Manzotti 2010</t>
+          <t>manzotti_2010</t>
         </is>
       </c>
       <c r="H17" t="n">
@@ -1599,6 +1639,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t>si</t>
@@ -1777,7 +1822,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Manzotti 2010</t>
+          <t>manzotti_2010</t>
         </is>
       </c>
       <c r="H22" t="n">
@@ -1850,6 +1895,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t>si</t>
@@ -1912,6 +1962,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t>si</t>
@@ -1974,6 +2029,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>sabatino_cap4</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
           <t>si</t>
@@ -2036,6 +2096,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t>si</t>
@@ -2098,6 +2163,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
           <t>si</t>
@@ -2160,6 +2230,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>sabatino_cap4</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr">
         <is>
           <t>si</t>
@@ -2222,6 +2297,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr">
         <is>
           <t>si</t>
@@ -2284,6 +2364,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
           <t>si</t>
@@ -2405,7 +2490,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Pinotti 2025</t>
+          <t>pinotti_2025</t>
         </is>
       </c>
       <c r="H32" t="n">
@@ -2478,6 +2563,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr">
         <is>
           <t>si</t>
@@ -2540,6 +2630,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr">
         <is>
           <t>si</t>
@@ -2602,6 +2697,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr">
         <is>
           <t>si</t>
@@ -2664,6 +2764,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr">
         <is>
           <t>si</t>
@@ -2783,6 +2888,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr">
         <is>
           <t>si</t>
@@ -2845,6 +2955,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
           <t>si</t>
@@ -2907,6 +3022,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
           <t>si</t>
@@ -2971,7 +3091,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Terzoli 2015</t>
+          <t>terzoli_2015</t>
         </is>
       </c>
       <c r="H41" t="n">
@@ -3039,6 +3159,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>sabatino_cap4</t>
+        </is>
+      </c>
       <c r="I42" t="inlineStr">
         <is>
           <t>si</t>
@@ -3101,6 +3226,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I43" t="inlineStr">
         <is>
           <t>si</t>
@@ -3163,6 +3293,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr">
         <is>
           <t>si</t>
@@ -3225,6 +3360,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I45" t="inlineStr">
         <is>
           <t>si</t>
@@ -3287,6 +3427,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>sabatino_cap4</t>
+        </is>
+      </c>
       <c r="I46" t="inlineStr">
         <is>
           <t>si</t>
@@ -3349,6 +3494,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I47" t="inlineStr">
         <is>
           <t>si</t>
@@ -3411,6 +3561,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I48" t="inlineStr">
         <is>
           <t>si</t>
@@ -3473,6 +3628,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I49" t="inlineStr">
         <is>
           <t>si</t>
@@ -3537,7 +3697,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Manzotti 2010</t>
+          <t>manzotti_2010</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -3607,6 +3767,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I51" t="inlineStr">
         <is>
           <t>si</t>
@@ -3671,7 +3836,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Cortellessa 2023</t>
+          <t>cortellessa_2023</t>
         </is>
       </c>
       <c r="H52" t="n">
@@ -3739,6 +3904,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>censimento_gaddatlas</t>
+        </is>
+      </c>
       <c r="I53" t="inlineStr">
         <is>
           <t>si</t>
@@ -3860,7 +4030,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Manzotti 2010</t>
+          <t>manzotti_2010</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -3937,7 +4107,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Manzotti 2010</t>
+          <t>manzotti_2010</t>
         </is>
       </c>
       <c r="H56" t="n">
@@ -4012,7 +4182,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Pinotti 2025</t>
+          <t>pinotti_2025</t>
         </is>
       </c>
       <c r="H57" t="n">
@@ -4087,7 +4257,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Terzoli 2015</t>
+          <t>terzoli_2015</t>
         </is>
       </c>
       <c r="H58" t="n">
@@ -4162,7 +4332,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Manzotti 2010</t>
+          <t>manzotti_2010</t>
         </is>
       </c>
       <c r="H59" t="n">
@@ -4237,7 +4407,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Manzotti 2010</t>
+          <t>manzotti_2010</t>
         </is>
       </c>
       <c r="H60" t="n">
@@ -4312,7 +4482,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Manzotti 2010</t>
+          <t>manzotti_2010</t>
         </is>
       </c>
       <c r="H61" t="n">
@@ -4387,7 +4557,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Manzotti 2010</t>
+          <t>manzotti_2010</t>
         </is>
       </c>
       <c r="H62" t="n">
@@ -4462,7 +4632,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Perosa 2023a</t>
+          <t>perosa_2023a</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -4534,12 +4704,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Lugnani, cit. in Perosa 2023a</t>
+          <t>perosa_2023a</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>104, n. 97</t>
+          <t>104, n. 97 (Lugnani 2001, cit.)</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4606,7 +4776,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Cortellessa 2023</t>
+          <t>cortellessa_2023</t>
         </is>
       </c>
       <c r="H65" t="n">
@@ -4676,7 +4846,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Perosa 2023a</t>
+          <t>perosa_2023a</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -4748,12 +4918,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Lugnani, cit. in Perosa 2023a</t>
+          <t>perosa_2023a</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>104, n. 97</t>
+          <t>104, n. 97 (Lugnani 2001, cit.)</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4820,7 +4990,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Cortellessa 2023</t>
+          <t>cortellessa_2023</t>
         </is>
       </c>
       <c r="H68" t="n">
@@ -4890,7 +5060,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Capitolo 4</t>
+          <t>sabatino_cap4</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -4962,7 +5132,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Censimento GaddAtlas</t>
+          <t>censimento_gaddatlas</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -5024,7 +5194,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Censimento GaddAtlas</t>
+          <t>censimento_gaddatlas</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -5086,7 +5256,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Censimento GaddAtlas</t>
+          <t>censimento_gaddatlas</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5148,7 +5318,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Manzotti 2010</t>
+          <t>manzotti_2010</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -5220,7 +5390,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>QP (Adelphi 2018)</t>
+          <t>qp</t>
         </is>
       </c>
       <c r="H74" t="n">
@@ -5285,7 +5455,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Pinotti 2025</t>
+          <t>pinotti_2025</t>
         </is>
       </c>
       <c r="H75" t="n">
@@ -5350,7 +5520,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Matt e Pinotti 2022</t>
+          <t>matt_pinotti_2022</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -5417,7 +5587,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Matt e Pinotti 2022</t>
+          <t>matt_pinotti_2022</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -5484,7 +5654,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>QP</t>
+          <t>qp</t>
         </is>
       </c>
       <c r="H78" t="n">
@@ -5554,7 +5724,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>QP</t>
+          <t>qp</t>
         </is>
       </c>
       <c r="H79" t="n">
@@ -5624,7 +5794,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>QP</t>
+          <t>qp</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -5691,7 +5861,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>QP</t>
+          <t>qp</t>
         </is>
       </c>
       <c r="H81" t="n">
@@ -5761,7 +5931,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>QP</t>
+          <t>qp</t>
         </is>
       </c>
       <c r="H82" t="n">
@@ -5826,7 +5996,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>QP</t>
+          <t>qp</t>
         </is>
       </c>
       <c r="H83" t="n">
@@ -5896,7 +6066,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>QP</t>
+          <t>qp</t>
         </is>
       </c>
       <c r="H84" t="n">
@@ -5966,7 +6136,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>QP</t>
+          <t>qp</t>
         </is>
       </c>
       <c r="H85" t="n">
@@ -6036,7 +6206,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>QP</t>
+          <t>qp</t>
         </is>
       </c>
       <c r="H86" t="n">
@@ -6106,7 +6276,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>QP</t>
+          <t>qp</t>
         </is>
       </c>
       <c r="H87" t="n">
@@ -6176,7 +6346,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>QP</t>
+          <t>qp</t>
         </is>
       </c>
       <c r="H88" t="n">
@@ -6246,7 +6416,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>QP</t>
+          <t>qp</t>
         </is>
       </c>
       <c r="H89" t="n">
@@ -6316,7 +6486,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>QP</t>
+          <t>qp</t>
         </is>
       </c>
       <c r="H90" t="n">
@@ -6386,7 +6556,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>QP</t>
+          <t>qp</t>
         </is>
       </c>
       <c r="H91" t="n">
@@ -6451,7 +6621,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>QP</t>
+          <t>qp</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -6518,7 +6688,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>QP</t>
+          <t>qp</t>
         </is>
       </c>
       <c r="H93" t="n">
@@ -6588,7 +6758,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>QP</t>
+          <t>qp</t>
         </is>
       </c>
       <c r="H94" t="n">
@@ -6653,7 +6823,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>QP</t>
+          <t>qp</t>
         </is>
       </c>
       <c r="H95" t="n">
@@ -6723,7 +6893,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>QP</t>
+          <t>qp</t>
         </is>
       </c>
       <c r="H96" t="n">
@@ -6793,7 +6963,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>QP</t>
+          <t>qp</t>
         </is>
       </c>
       <c r="H97" t="n">
@@ -6863,7 +7033,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>QP</t>
+          <t>qp</t>
         </is>
       </c>
       <c r="H98" t="n">

</xml_diff>

<commit_message>
posizioni attribuite: LocationAssertion per Casal Bruciato (B3, D-069)
L-0001 (TCI, adottata) e L-0002 (IGM) di Manzotti 2010 su
gaz_casale_abbruciato: geometria WKT, repertorio datato, precisione,
datum (Locations.tsv). IQ19: coordinata dell'entità = posizione adottata.
Authority_Source ridotto a rinvio. Shape 21.
TBox 1.422 -> 1.444, ABox 38.588 -> 38.668.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Assertions.xlsx
+++ b/data/source/xlsx/Assertions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q98"/>
+  <dimension ref="A1:Q100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7070,6 +7070,150 @@
         </is>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>L-0001</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_casale_abbruciato</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>geometry/L-0001</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>manzotti</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>manzotti_2010</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>268–269; Tavv. VI–VII, pp. 300–301</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>La carta TCI colloca il casale fra le ferrovie Roma–Velletri e Roma–Napoli, all'altezza di Santa Fumia, lungo il fosso di Casale Abbrusciato, come il testo. Coordinate stimate: punto mediano fra le due ferrovie alla latitudine di Borgo Santa Fumia.</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>Posizione adottata (D-037).</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>L-0002</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_casale_abbruciato</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>geometry/L-0002</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>manzotti</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>manzotti_2010</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>268–269; Tavv. VI–VII, pp. 300–301</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>La tavoletta IGM colloca «Casale Abbruciato» a ovest della Roma–Napoli: reticolo UTM 33 della tavola, E 297,7 N 4621,3 km.</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>Posizione alternativa (D-037).</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
l'occorrenza come primitiva: fondamento, varianti, memoria, incertezza (B4, D-070)
chora:groundedIn (esplicito o di default, 764 triple); varianti da
occorrenza QP a occorrenza dell'altro testimone (6, con QPL 285 <-> QP 16,
293 <-> 25); memoria e incertezza sul nome sull'occorrenza; adozione
scritta su tutte le interpretazioni; adapter solo sulle adottate.
ReifiedTypeShape (SHACL-SPARQL), shape 22, IQ18, IQ20 (avvertenza: 6
terne in TERNE_IQ20.md).
TBox 1.444 -> 1.459, ABox 38.668 -> 40.459, SHACL conforme (50).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Assertions.xlsx
+++ b/data/source/xlsx/Assertions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q100"/>
+  <dimension ref="A1:R102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -502,6 +502,11 @@
           <t>Uncertainty_Origin</t>
         </is>
       </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Grounded_In</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -569,6 +574,11 @@
           <t>validata</t>
         </is>
       </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>ref_00651</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -639,6 +649,11 @@
           <t>validata</t>
         </is>
       </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>ref_00651</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1550,6 +1565,11 @@
           <t>validata</t>
         </is>
       </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>ref_00651</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4010,7 +4030,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>narrativeplace/casal_bruciato</t>
+          <t>gazetteer/gaz_casale_abbruciato</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -4148,6 +4168,11 @@
           <t>costruttiva</t>
         </is>
       </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>ref_00651</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4223,6 +4248,11 @@
           <t>documentaria</t>
         </is>
       </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>ref_00435</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4237,7 +4267,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>narrativeplace/robine_vecchie</t>
+          <t>reference/ref_00403</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -4312,7 +4342,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>narrativeplace/edicola_due_santi</t>
+          <t>gazetteer/gaz_edicola_due_santi</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -4448,6 +4478,11 @@
           <t>documentaria</t>
         </is>
       </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>ref_00541</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4462,7 +4497,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>narrativeplace/carsoli</t>
+          <t>reference/ref_00523</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -4598,6 +4633,11 @@
           <t>documentaria</t>
         </is>
       </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>ref_00535|ref_00635|ref_00703</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4612,7 +4652,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>interpretation/interp_00168</t>
+          <t>reference/ref_00144</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -4684,7 +4724,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>interpretation/interp_00168</t>
+          <t>reference/ref_00144</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -4756,7 +4796,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>interpretation/interp_00168</t>
+          <t>reference/ref_00144</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -4826,7 +4866,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>interpretation/interp_00169</t>
+          <t>reference/ref_00145</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -4898,7 +4938,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>interpretation/interp_00169</t>
+          <t>reference/ref_00145</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -4970,7 +5010,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>interpretation/interp_00169</t>
+          <t>reference/ref_00145</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -5370,12 +5410,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>narrativeplace/frattocchie</t>
+          <t>reference/ref_00588</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>reference/ref_00588|reference/ref_00724</t>
+          <t>reference/ref_00724</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -5435,12 +5475,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>narrativeplace/via_lanza</t>
+          <t>reference/ref_00436</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>reference/ref_00436|reference/ref_00725</t>
+          <t>reference/ref_00725</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -5490,7 +5530,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>V-0003</t>
+          <t>V-0003a</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -5500,12 +5540,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>narrativeplace/palazzo_219</t>
+          <t>reference/ref_00007</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>reference/ref_00007|reference/ref_00036|reference/ref_00726|reference/ref_00727</t>
+          <t>reference/ref_00726</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -5530,7 +5570,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>Civico 119 (QPL 285, 293: «quer gran palazzo del centodicinnove») / 219 (QP 16, 25: «ducentodicinnove»): il palazzo si ricolloca solo nell'edizione in volume.</t>
+          <t>Civico 119 (QPL 285) / 219 (QP 16).</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
@@ -5540,7 +5580,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>Cap. 4, § 4.2 (r. 45).</t>
+          <t>Corrispondenza QPL 285 ↔ QP 16 confermata da LS (9/10/2026). Cap. 4, § 4.2 (r. 45).</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
@@ -5557,7 +5597,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>V-0004</t>
+          <t>V-0003b</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -5567,12 +5607,12 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>narrativeplace/palazzo_219</t>
+          <t>reference/ref_00036</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>reference/ref_00008|reference/ref_00038|reference/ref_00726|reference/ref_00727</t>
+          <t>reference/ref_00727</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -5597,7 +5637,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>«palazzo degli ori» (QPL 285, 293) / «palazzo dell'Oro» (QP 16, 25).</t>
+          <t>Civico 119 (QPL 293) / 219 (QP 25).</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
@@ -5607,7 +5647,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>Cap. 4, § 4.2 (r. 45).</t>
+          <t>Corrispondenza QPL 293 ↔ QP 25 confermata da LS (9/10/2026). Cap. 4, § 4.2 (r. 45).</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
@@ -5624,50 +5664,47 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>R-0001</t>
+          <t>V-0004a</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>route</t>
+          <t>variant</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>route/tragitto_torraccio_ponte_divino_amore</t>
+          <t>reference/ref_00008</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>chora:CompletedRoute</t>
+          <t>reference/ref_00726</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
+          <t>matt|pinotti</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
           <t>lorenzo_sabatino</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>lorenzo_sabatino</t>
-        </is>
-      </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>qp</t>
-        </is>
-      </c>
-      <c r="H78" t="n">
-        <v>297</v>
-      </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>si</t>
+          <t>matt_pinotti_2022</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>schede 8, 11, 30, 31</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>«Discesero ai Torraccio […] Svoltarono sull'Appia a li Due Santi […] Valicò invece il binario»: Ingravallo, Di Pietrantonio, l'autista e Runzato percorrono il tragitto in auto.</t>
+          <t>«palazzo degli ori» (QPL 285) / «palazzo dell'Oro» (QP 16).</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
@@ -5677,7 +5714,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>L'ultimo nodo (ponte del Divino Amore) è un termine di paragone («simile a quello ch'era due chilometri più a nord, presso il ponte»): lasciato invariato per decisione di LS (9/10/2026, D-064).</t>
+          <t>Corrispondenza QPL 285 ↔ QP 16 confermata da LS (9/10/2026). Cap. 4, § 4.2 (r. 45).</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -5687,57 +5724,54 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>R-0002</t>
+          <t>V-0004b</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>route</t>
+          <t>variant</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>route/tragitto_santarella_torraccio_divino_amore</t>
+          <t>reference/ref_00038</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>chora:InferredRoute</t>
+          <t>reference/ref_00727</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
+          <t>matt|pinotti</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
           <t>lorenzo_sabatino</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>lorenzo_sabatino</t>
-        </is>
-      </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>qp</t>
-        </is>
-      </c>
-      <c r="H79" t="n">
-        <v>169</v>
-      </c>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t>si</t>
+          <t>matt_pinotti_2022</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>schede 8, 11, 30, 31</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>La motocicletta di Santarella «si preannunciava di lontano, dal Torraccio, […] o dal Divino Amore»: le provenienze si ricavano dal rumore, «altre volte» da un luogo o dall'altro.</t>
+          <t>«palazzo degli ori» (QPL 293) / «palazzo dell'Oro» (QP 25).</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
@@ -5747,7 +5781,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>Separato dal tragitto di QP 297 (D-060). È un elenco disgiuntivo e abituale di provenienze, non una sequenza: potrebbe non essere un percorso.</t>
+          <t>Corrispondenza QPL 293 ↔ QP 25 confermata da LS (9/10/2026). Cap. 4, § 4.2 (r. 45).</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -5757,14 +5791,14 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>R-0003</t>
+          <t>R-0001</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -5774,7 +5808,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>route/tragitto_tenenza_due_santi</t>
+          <t>route/tragitto_torraccio_ponte_divino_amore</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -5797,10 +5831,8 @@
           <t>qp</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr">
-        <is>
-          <t>208–215</t>
-        </is>
+      <c r="H80" t="n">
+        <v>297</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
@@ -5809,12 +5841,17 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>Pestalozzi e Cocullo scendono dalla caserma di Marino alla porta del borgo, prendono l'Appia, passano la Fontana e si fermano ai Due Santi.</t>
+          <t>«Discesero ai Torraccio […] Svoltarono sull'Appia a li Due Santi […] Valicò invece il binario»: Ingravallo, Di Pietrantonio, l'autista e Runzato percorrono il tragitto in auto.</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
         <is>
           <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>L'ultimo nodo (ponte del Divino Amore) è un termine di paragone («simile a quello ch'era due chilometri più a nord, presso il ponte»): lasciato invariato per decisione di LS (9/10/2026, D-064).</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -5831,7 +5868,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>R-0004</t>
+          <t>R-0002</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -5841,12 +5878,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>route/tragitto_brancaccio_piazza_san_giovanni</t>
+          <t>route/tragitto_santarella_torraccio_divino_amore</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>chora:CompletedRoute</t>
+          <t>chora:InferredRoute</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -5865,7 +5902,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>292</v>
+        <v>169</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
@@ -5874,7 +5911,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>«A largo Brancaccio, mentre che staveno svortando in via Merulana verso piazza San Giovanni»: il tragitto è in corso.</t>
+          <t>La motocicletta di Santarella «si preannunciava di lontano, dal Torraccio, […] o dal Divino Amore»: le provenienze si ricavano dal rumore, «altre volte» da un luogo o dall'altro.</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
@@ -5884,7 +5921,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>L'ultimo nodo è una direzione («verso piazza San Giovanni»): l'arrivo non è narrato.</t>
+          <t>Separato dal tragitto di QP 297 (D-060). È un elenco disgiuntivo e abituale di provenienze, non una sequenza: potrebbe non essere un percorso.</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -5901,7 +5938,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>R-0005</t>
+          <t>R-0003</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -5911,7 +5948,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>route/tragitto_viminale_merulana</t>
+          <t>route/tragitto_tenenza_due_santi</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -5934,8 +5971,10 @@
           <t>qp</t>
         </is>
       </c>
-      <c r="H82" t="n">
-        <v>25</v>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>208–215</t>
+        </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
@@ -5944,7 +5983,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>«Saliti sul PV e discesi appunto al Viminale, presero il tram di San Giovanni […] raggiunsero il civico ducentodicinnove».</t>
+          <t>Pestalozzi e Cocullo scendono dalla caserma di Marino alla porta del borgo, prendono l'Appia, passano la Fontana e si fermano ai Due Santi.</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
@@ -5966,7 +6005,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>R-0006</t>
+          <t>R-0004</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -5976,12 +6015,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>route/tragitto_appia_falcognana</t>
+          <t>route/tragitto_brancaccio_piazza_san_giovanni</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>chora:IndicatedRoute</t>
+          <t>chora:CompletedRoute</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -6000,7 +6039,7 @@
         </is>
       </c>
       <c r="H83" t="n">
-        <v>238</v>
+        <v>292</v>
       </c>
       <c r="I83" t="inlineStr">
         <is>
@@ -6009,7 +6048,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>«La strada era una sola, pe fortuna, salvo il primo pezzo però: la statale, l'Appia, poi ad angolo retto la deviazione della provinciale, pe Falcognana»: la strada spiegata dopo le indicazioni di Camilla (QP 237).</t>
+          <t>«A largo Brancaccio, mentre che staveno svortando in via Merulana verso piazza San Giovanni»: il tragitto è in corso.</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
@@ -6019,7 +6058,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>Incerto fra indicato e compiuto: il passo descrive la strada, il viaggio segue.</t>
+          <t>L'ultimo nodo è una direzione («verso piazza San Giovanni»): l'arrivo non è narrato.</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -6036,7 +6075,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>R-0007</t>
+          <t>R-0005</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -6046,7 +6085,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>route/tragitto_agostino_aquiro</t>
+          <t>route/tragitto_viminale_merulana</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -6070,7 +6109,7 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
@@ -6079,17 +6118,12 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>Il commendator Angeloni e i suoi pari «sogliono deambulare» da Sant'Agostino a Santa Maria in Aquiro.</t>
+          <t>«Saliti sul PV e discesi appunto al Viminale, presero il tram di San Giovanni […] raggiunsero il civico ducentodicinnove».</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
         <is>
           <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="M84" t="inlineStr">
-        <is>
-          <t>Percorso abituale (iterativo).</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -6106,7 +6140,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>R-0008</t>
+          <t>R-0006</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -6116,12 +6150,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>route/tragitto_cecchina_anziate</t>
+          <t>route/tragitto_appia_falcognana</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>chora:CompletedRoute</t>
+          <t>chora:IndicatedRoute</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -6140,7 +6174,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>173</v>
+        <v>238</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
@@ -6149,7 +6183,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>La motocicletta di Santarella «infilava […] la mala curva d'aa stazione d'aa Cecchina», poi si fermava a Santa Palomba e a Campoleone, «il caso richiedendo».</t>
+          <t>«La strada era una sola, pe fortuna, salvo il primo pezzo però: la statale, l'Appia, poi ad angolo retto la deviazione della provinciale, pe Falcognana»: la strada spiegata dopo le indicazioni di Camilla (QP 237).</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
@@ -6159,7 +6193,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>Percorso abituale (iterativo), con fermate eventuali.</t>
+          <t>Incerto fra indicato e compiuto: il passo descrive la strada, il viaggio segue.</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -6176,7 +6210,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>R-0009</t>
+          <t>R-0007</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -6186,7 +6220,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>route/tragitto_colonna_treccani</t>
+          <t>route/tragitto_agostino_aquiro</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -6219,7 +6253,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>Angeloni e i suoi pari «si avventurano» per via Colonna, piazza de Pietra, via de Pietra fino al Corso.</t>
+          <t>Il commendator Angeloni e i suoi pari «sogliono deambulare» da Sant'Agostino a Santa Maria in Aquiro.</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
@@ -6246,7 +6280,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>R-0010</t>
+          <t>R-0008</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -6256,12 +6290,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>route/tragitto_frattocchie_ciampino</t>
+          <t>route/tragitto_cecchina_anziate</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>chora:InferredRoute</t>
+          <t>chora:CompletedRoute</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -6280,7 +6314,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
@@ -6289,7 +6323,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>«Oppure a metà le Frattocchie, doveva spengere: al passaggio dell'Appia, o a Ca' Francesi, a Tor Ser Paolo, alla stazione di Ciampino»: luoghi alternativi della fermata.</t>
+          <t>La motocicletta di Santarella «infilava […] la mala curva d'aa stazione d'aa Cecchina», poi si fermava a Santa Palomba e a Campoleone, «il caso richiedendo».</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
@@ -6299,7 +6333,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>Come QP 169: elenco disgiuntivo e abituale, non una sequenza.</t>
+          <t>Percorso abituale (iterativo), con fermate eventuali.</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -6316,7 +6350,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>R-0011</t>
+          <t>R-0009</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -6326,7 +6360,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>route/tragitto_monti_piazza_esedra</t>
+          <t>route/tragitto_colonna_treccani</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -6350,7 +6384,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>182</v>
+        <v>40</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
@@ -6359,7 +6393,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>Diomede «si differiva passo passo da un quartiere all'altro: monticiano a le dieci, trasteverino a le quattro, a Piazza Colonna o a l'Esedra».</t>
+          <t>Angeloni e i suoi pari «si avventurano» per via Colonna, piazza de Pietra, via de Pietra fino al Corso.</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
@@ -6369,7 +6403,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>Percorso abituale (iterativo); l'ultimo nodo è disgiuntivo («o»).</t>
+          <t>Percorso abituale (iterativo).</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -6386,7 +6420,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>R-0012</t>
+          <t>R-0010</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -6396,12 +6430,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>route/tragitto_rocca_di_papa_monte_nuncupale</t>
+          <t>route/tragitto_frattocchie_ciampino</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>chora:CompletedRoute</t>
+          <t>chora:InferredRoute</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -6420,7 +6454,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
@@ -6429,7 +6463,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>Santarella «da Rocca di Papa a Castel Savelli, giù: da Rocca Orsina al Monte Nuncupale, su».</t>
+          <t>«Oppure a metà le Frattocchie, doveva spengere: al passaggio dell'Appia, o a Ca' Francesi, a Tor Ser Paolo, alla stazione di Ciampino»: luoghi alternativi della fermata.</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
@@ -6439,7 +6473,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>Percorso abituale (iterativo).</t>
+          <t>Come QP 169: elenco disgiuntivo e abituale, non una sequenza.</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -6456,7 +6490,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>R-0013</t>
+          <t>R-0011</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -6466,7 +6500,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>route/tragitto_chiara_pantheon</t>
+          <t>route/tragitto_monti_piazza_esedra</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -6490,7 +6524,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>41</v>
+        <v>182</v>
       </c>
       <c r="I90" t="inlineStr">
         <is>
@@ -6499,7 +6533,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>Di quaresima Angeloni e i suoi pari «si contentano lungheggiar Santa Chiara […] imboccheno la Palommella e sfioreno er dedietro ar Panteone».</t>
+          <t>Diomede «si differiva passo passo da un quartiere all'altro: monticiano a le dieci, trasteverino a le quattro, a Piazza Colonna o a l'Esedra».</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
@@ -6509,7 +6543,7 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>Percorso abituale (iterativo).</t>
+          <t>Percorso abituale (iterativo); l'ultimo nodo è disgiuntivo («o»).</t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
@@ -6526,7 +6560,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>R-0014</t>
+          <t>R-0012</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -6536,7 +6570,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>route/tragitto_duesanti_frattocchie</t>
+          <t>route/tragitto_rocca_di_papa_monte_nuncupale</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -6560,7 +6594,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>56</v>
+        <v>173</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
@@ -6569,12 +6603,17 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>La corsa del tram dei Castelli: «Ai Due Santi, al Torraccio, a le Frattocchie […] era salita una quantità di persone».</t>
+          <t>Santarella «da Rocca di Papa a Castel Savelli, giù: da Rocca Orsina al Monte Nuncupale, su».</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
         <is>
           <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>Percorso abituale (iterativo).</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
@@ -6591,7 +6630,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>R-0015</t>
+          <t>R-0013</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -6601,7 +6640,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>route/tragitto_policlinico_san_lorenzo_al_verano</t>
+          <t>route/tragitto_chiara_pantheon</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -6624,10 +6663,8 @@
           <t>qp</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr">
-        <is>
-          <t>139–140</t>
-        </is>
+      <c r="H92" t="n">
+        <v>41</v>
       </c>
       <c r="I92" t="inlineStr">
         <is>
@@ -6636,12 +6673,17 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>Il corteo funebre «spostò dar Policlinico a le otto […] tajarono pe la direttissima der viale Regina Margherita […] arrivarono a San Lorenzo ar Verano».</t>
+          <t>Di quaresima Angeloni e i suoi pari «si contentano lungheggiar Santa Chiara […] imboccheno la Palommella e sfioreno er dedietro ar Panteone».</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
         <is>
           <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>Percorso abituale (iterativo).</t>
         </is>
       </c>
       <c r="N92" t="inlineStr">
@@ -6658,7 +6700,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>R-0016</t>
+          <t>R-0014</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -6668,12 +6710,12 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>route/tragitto_marino_albano_laziale</t>
+          <t>route/tragitto_duesanti_frattocchie</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>chora:DirectionalRoute</t>
+          <t>chora:CompletedRoute</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -6692,7 +6734,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>278</v>
+        <v>56</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
@@ -6701,17 +6743,12 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>Santarella «era a percorrere sulla sua motocicletta la via provinciale da Marino ad Albano»: il passo dà la strada e la sua direzione, non il tratto percorso.</t>
+          <t>La corsa del tram dei Castelli: «Ai Due Santi, al Torraccio, a le Frattocchie […] era salita una quantità di persone».</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
         <is>
           <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="M93" t="inlineStr">
-        <is>
-          <t>Alternativa: compiuto. Il Cap. 4 (r. 194) chiama questo tipo «presunto».</t>
         </is>
       </c>
       <c r="N93" t="inlineStr">
@@ -6728,7 +6765,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>R-0017</t>
+          <t>R-0015</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -6738,7 +6775,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>route/tragitto_marino_due_santi</t>
+          <t>route/tragitto_policlinico_san_lorenzo_al_verano</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -6761,8 +6798,10 @@
           <t>qp</t>
         </is>
       </c>
-      <c r="H94" t="n">
-        <v>206</v>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>139–140</t>
+        </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
@@ -6771,7 +6810,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>Pestalozzi «usciva (in motocicletta) dalla caserma […] di Marino per catapultarsi alla bottega-laboratorio».</t>
+          <t>Il corteo funebre «spostò dar Policlinico a le otto […] tajarono pe la direttissima der viale Regina Margherita […] arrivarono a San Lorenzo ar Verano».</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
@@ -6793,7 +6832,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>R-0018</t>
+          <t>R-0016</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -6803,12 +6842,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>route/tragitto_marino_santo_stefano</t>
+          <t>route/tragitto_marino_albano_laziale</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>chora:CompletedRoute</t>
+          <t>chora:DirectionalRoute</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -6827,7 +6866,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>153</v>
+        <v>278</v>
       </c>
       <c r="I95" t="inlineStr">
         <is>
@@ -6836,7 +6875,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>«arrivò a Santo Stefano in motocicletta il brigadiere Pestalozzi […] latore di un rapporto […] della Tenenza».</t>
+          <t>Santarella «era a percorrere sulla sua motocicletta la via provinciale da Marino ad Albano»: il passo dà la strada e la sua direzione, non il tratto percorso.</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">
@@ -6846,7 +6885,7 @@
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>Nodi nell'ordine di occorrenza nel testo (decisione di LS, 9/10/2026, D-064): Santo Stefano 1, Tenenza 2. La partenza dalla Tenenza è inferita dal rapporto.</t>
+          <t>Alternativa: compiuto. Il Cap. 4 (r. 194) chiama questo tipo «presunto».</t>
         </is>
       </c>
       <c r="N95" t="inlineStr">
@@ -6863,7 +6902,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>R-0019</t>
+          <t>R-0017</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -6873,7 +6912,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>route/tragitto_merulana_policlinico</t>
+          <t>route/tragitto_marino_due_santi</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -6897,7 +6936,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>93</v>
+        <v>206</v>
       </c>
       <c r="I96" t="inlineStr">
         <is>
@@ -6906,17 +6945,12 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>L'autorità giudiziaria «era intervenuta […] a via Merulana, indi al Policlinico».</t>
+          <t>Pestalozzi «usciva (in motocicletta) dalla caserma […] di Marino per catapultarsi alla bottega-laboratorio».</t>
         </is>
       </c>
       <c r="L96" t="inlineStr">
         <is>
           <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="M96" t="inlineStr">
-        <is>
-          <t>Focalizzatrice del tragitto: Liliana, come nel database (decisione di LS, 9/10/2026, D-064).</t>
         </is>
       </c>
       <c r="N96" t="inlineStr">
@@ -6933,7 +6967,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>R-0020</t>
+          <t>R-0018</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -6943,12 +6977,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>route/tragitto_sogno_casal_bruciato_campo_morto</t>
+          <t>route/tragitto_marino_santo_stefano</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>chora:DreamedRoute</t>
+          <t>chora:CompletedRoute</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -6967,7 +7001,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>212</v>
+        <v>153</v>
       </c>
       <c r="I97" t="inlineStr">
         <is>
@@ -6976,7 +7010,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>Il sogno di Pestalozzi: «al passaggio a livello di Casal Bruciato il vetrone girasole... per fil a dest!», il Roma-Napoli che «filava filava», la fuga «verso le gore senza foce del Campo Morto».</t>
+          <t>«arrivò a Santo Stefano in motocicletta il brigadiere Pestalozzi […] latore di un rapporto […] della Tenenza».</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
@@ -6986,7 +7020,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>Nuovo percorso (D-060). La lettura di Manzotti di «per fil a dest» (2010, p. 269) è una nota attribuita di fase 3.</t>
+          <t>Nodi nell'ordine di occorrenza nel testo (decisione di LS, 9/10/2026, D-064): Santo Stefano 1, Tenenza 2. La partenza dalla Tenenza è inferita dal rapporto.</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -7003,7 +7037,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>R-0021</t>
+          <t>R-0019</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -7013,12 +7047,12 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>route/tragitto_castel_di_leva_casal_bruciato</t>
+          <t>route/tragitto_merulana_policlinico</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>chora:IndicatedRoute</t>
+          <t>chora:CompletedRoute</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -7037,7 +7071,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>237</v>
+        <v>93</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
@@ -7046,7 +7080,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>Camilla indica la strada: «Pe la strada de Castel de Leva, fino ar ponte: poi, a sinistra, fino ar passaggio a livello de Casal Bruciato».</t>
+          <t>L'autorità giudiziaria «era intervenuta […] a via Merulana, indi al Policlinico».</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -7056,7 +7090,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>Nuovo percorso (D-060). Il nodo finale è il passaggio a livello: nei dati l'occorrenza è di casal_bruciato.</t>
+          <t>Focalizzatrice del tragitto: Liliana, come nel database (decisione di LS, 9/10/2026, D-064).</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -7073,27 +7107,27 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>L-0001</t>
+          <t>R-0020</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>route</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>gazetteer/gaz_casale_abbruciato</t>
+          <t>route/tragitto_sogno_casal_bruciato_campo_morto</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>geometry/L-0001</t>
+          <t>chora:DreamedRoute</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>manzotti</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -7103,13 +7137,11 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>manzotti_2010</t>
-        </is>
-      </c>
-      <c r="H99" t="inlineStr">
-        <is>
-          <t>268–269; Tavv. VI–VII, pp. 300–301</t>
-        </is>
+          <t>qp</t>
+        </is>
+      </c>
+      <c r="H99" t="n">
+        <v>212</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
@@ -7118,7 +7150,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>La carta TCI colloca il casale fra le ferrovie Roma–Velletri e Roma–Napoli, all'altezza di Santa Fumia, lungo il fosso di Casale Abbrusciato, come il testo. Coordinate stimate: punto mediano fra le due ferrovie alla latitudine di Borgo Santa Fumia.</t>
+          <t>Il sogno di Pestalozzi: «al passaggio a livello di Casal Bruciato il vetrone girasole... per fil a dest!», il Roma-Napoli che «filava filava», la fuga «verso le gore senza foce del Campo Morto».</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
@@ -7128,87 +7160,229 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>Posizione adottata (D-037).</t>
+          <t>Nuovo percorso (D-060). La lettura di Manzotti di «per fil a dest» (2010, p. 269) è una nota attribuita di fase 3.</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
         <is>
-          <t>prova referenziale</t>
+          <t>prova testuale</t>
         </is>
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>validata</t>
+          <t>bozza</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
+          <t>R-0021</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>route/tragitto_castel_di_leva_casal_bruciato</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>chora:IndicatedRoute</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>qp</t>
+        </is>
+      </c>
+      <c r="H100" t="n">
+        <v>237</v>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Camilla indica la strada: «Pe la strada de Castel de Leva, fino ar ponte: poi, a sinistra, fino ar passaggio a livello de Casal Bruciato».</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>Nuovo percorso (D-060). Il nodo finale è il passaggio a livello: nei dati l'occorrenza è di casal_bruciato.</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>bozza</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>L-0001</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_casale_abbruciato</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>geometry/L-0001</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>manzotti</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>manzotti_2010</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>268–269; Tavv. VI–VII, pp. 300–301</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>La carta TCI colloca il casale fra le ferrovie Roma–Velletri e Roma–Napoli, all'altezza di Santa Fumia, lungo il fosso di Casale Abbrusciato, come il testo. Coordinate stimate: punto mediano fra le due ferrovie alla latitudine di Borgo Santa Fumia.</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>Posizione adottata (D-037).</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
           <t>L-0002</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr">
+      <c r="B102" t="inlineStr">
         <is>
           <t>location</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr">
+      <c r="C102" t="inlineStr">
         <is>
           <t>gazetteer/gaz_casale_abbruciato</t>
         </is>
       </c>
-      <c r="D100" t="inlineStr">
+      <c r="D102" t="inlineStr">
         <is>
           <t>geometry/L-0002</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr">
+      <c r="E102" t="inlineStr">
         <is>
           <t>manzotti</t>
         </is>
       </c>
-      <c r="F100" t="inlineStr">
+      <c r="F102" t="inlineStr">
         <is>
           <t>lorenzo_sabatino</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr">
+      <c r="G102" t="inlineStr">
         <is>
           <t>manzotti_2010</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr">
+      <c r="H102" t="inlineStr">
         <is>
           <t>268–269; Tavv. VI–VII, pp. 300–301</t>
         </is>
       </c>
-      <c r="I100" t="inlineStr">
+      <c r="I102" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J100" t="inlineStr">
+      <c r="J102" t="inlineStr">
         <is>
           <t>La tavoletta IGM colloca «Casale Abbruciato» a ovest della Roma–Napoli: reticolo UTM 33 della tavola, E 297,7 N 4621,3 km.</t>
         </is>
       </c>
-      <c r="L100" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="M100" t="inlineStr">
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
         <is>
           <t>Posizione alternativa (D-037).</t>
         </is>
       </c>
-      <c r="N100" t="inlineStr">
+      <c r="N102" t="inlineStr">
         <is>
           <t>prova referenziale</t>
         </is>
       </c>
-      <c r="O100" t="inlineStr">
+      <c r="O102" t="inlineStr">
         <is>
           <t>validata</t>
         </is>

</xml_diff>

<commit_message>
correzioni: Lugnani 2001, due statuti validati, motivazione dei generati (D-071)
Atto di Lugnani datato 2001 (chora:originalSource), estratto da Perosa
2023a; S-casal_bruciato e S-edicola_due_santi validate (avvertenze 50 ->
48); statuti generati: «referente identificato nel gazetteer del
progetto». Prefissi hico e cito nel TTL.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Assertions.xlsx
+++ b/data/source/xlsx/Assertions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R102"/>
+  <dimension ref="A1:S102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,6 +507,11 @@
           <t>Grounded_In</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Original_Source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1286,7 +1291,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Statuto deciso e motivato da LS: D-029, D-037. Validata (D-071).</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1296,7 +1301,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1870,7 +1875,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Statuto deciso e motivato da LS: D-031. Validata (D-071).</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1880,7 +1885,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -4749,7 +4754,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>104, n. 97 (Lugnani 2001, cit.)</t>
+          <t>104, n. 97</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4769,7 +4774,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>Cap. 4, § 4.3: le tre letture convivono, nessuna è adottata dal progetto.</t>
+          <t>Cap. 4, § 4.3: le tre letture convivono, nessuna è adottata dal progetto. Lugnani 2001, cit. in Perosa 2023a, p. 104, n. 97.</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -4780,6 +4785,11 @@
       <c r="O64" t="inlineStr">
         <is>
           <t>bozza</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>lugnani_2001</t>
         </is>
       </c>
     </row>
@@ -4963,7 +4973,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>104, n. 97 (Lugnani 2001, cit.)</t>
+          <t>104, n. 97</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4983,7 +4993,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>Cap. 4, § 4.3: le tre letture convivono, nessuna è adottata dal progetto.</t>
+          <t>Cap. 4, § 4.3: le tre letture convivono, nessuna è adottata dal progetto. Lugnani 2001, cit. in Perosa 2023a, p. 104, n. 97.</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -4994,6 +5004,11 @@
       <c r="O67" t="inlineStr">
         <is>
           <t>bozza</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>lugnani_2001</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
terne di IQ20: cinque risolte, Cassero fermo, censimento (D-072)
via delle Oche a Bologna (U-0009, traslazione d'autore); Tevere/Biferno
un'interpretazione con due ancore e Between; via Nicotera divisa in due
occorrenze (ref_00730); Aliciaro e bivio con ancoraggi relazionali tipizzati
(tipo:id). Cassero fermo: manca l'entità di Sant'Ignazio. Censimento: 7
estratti con toponimo ripetuto, in TERNE_IQ20.md. IQ20 = 1, avvertenza.
Interpretazioni 961 -> 956.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Assertions.xlsx
+++ b/data/source/xlsx/Assertions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S102"/>
+  <dimension ref="A1:S103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7403,6 +7403,78 @@
         </is>
       </c>
     </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>U-0009</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>uncertainty</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_bologna</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>chora:Discrepancy</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>Il testo colloca a Milano ("udito a Milano […] al dispensario celtico di via delle Oche") la via bolognese delle Oche, nota via di prostituzione: traslazione d'autore, registrata e non corretta.</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>Luogo: via_delle_oche (QP 22). Soggetto l'entità dell'ancora, per la regola dell'asse geometria (D-070); lo statuto del luogo non cambia (D-072).</t>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>geometria</t>
+        </is>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>documentaria</t>
+        </is>
+      </c>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>ref_00028</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
sigle dei testimoni: QPL, QP, QPa (D-073)
QPa = Adelphi 2018 (witness/qpa, prefLabel «QP (Adelphi 2018)»),
testimone di riferimento di 726 occorrenze; QP = versione in volume 1957
(QP57 fuso, witness/qp cambia significato); RR II diventa una fonte in cui
QPL e QP sono letti (chora:readIn). V-0001 e ref_00724 su QP. «QP n» ->
«QPa n» nei campi dei dati, fuori dalle citazioni del Cap. 4. Il pannello
del testo legge witnessLabel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Assertions.xlsx
+++ b/data/source/xlsx/Assertions.xlsx
@@ -556,7 +556,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Lettura del censimento: la «stazione di Castello» (QP 279) come Castel Gandolfo, lettura immediata del toponimo. Identificazione contesa (DC-04): Manzotti 2010, p. 293 legge Castel Savello; la sua lettura entra in fase 3. Non adottata finché DC-04 non è deciso.</t>
+          <t>Lettura del censimento: la «stazione di Castello» (QPa 279) come Castel Gandolfo, lettura immediata del toponimo. Identificazione contesa (DC-04): Manzotti 2010, p. 293 legge Castel Savello; la sua lettura entra in fase 3. Non adottata finché DC-04 non è deciso.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>La «stazione di Castello» (QP 279) è la stazione dei carabinieri di Castel Savello: Manzotti scioglie così la dizione, contro la lettura immediata Castel Gandolfo (Cap. 4, § 4.4). Lettura adottata dal progetto (LS, 9/10/2026, DC-04).</t>
+          <t>La «stazione di Castello» (QPa 279) è la stazione dei carabinieri di Castel Savello: Manzotti scioglie così la dizione, contro la lettura immediata Castel Gandolfo (Cap. 4, § 4.4). Lettura adottata dal progetto (LS, 9/10/2026, DC-04).</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>La «stazione di Castello» (QP 279) è la stazione dei carabinieri di Castel Savello: identificazione adottata A-0002 (Manzotti 2010, p. 293). Il luogo testuale nomina in forma ellittica un luogo reale: statuto Imported. La lettura alternativa (Castel Gandolfo, A-0001) è anch'essa un luogo reale.</t>
+          <t>La «stazione di Castello» (QPa 279) è la stazione dei carabinieri di Castel Savello: identificazione adottata A-0002 (Manzotti 2010, p. 293). Il luogo testuale nomina in forma ellittica un luogo reale: statuto Imported. La lettura alternativa (Castel Gandolfo, A-0001) è anch'essa un luogo reale.</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -2401,7 +2401,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Statuto Transformed confermato da LS (D-035, 9/10/2026). Cap. 4, tab. 4.2 (r. 273): «Palazzo al 219» come caso generatore di R07; DATA_CHECKS DC-08: edificio in una via reale, Transformed salvo diversa evidenza. Varianti 119 → 219 (QPL 285, 293 / QP 16, 25) in fase 2 (T-41).</t>
+          <t>Statuto Transformed confermato da LS (D-035, 9/10/2026). Cap. 4, tab. 4.2 (r. 273): «Palazzo al 219» come caso generatore di R07; DATA_CHECKS DC-08: edificio in una via reale, Transformed salvo diversa evidenza. Varianti 119 → 219 (QPL 285, 293 / QPa 16, 25) in fase 2 (T-41).</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Palazzo reale (Simonetti o De Carolis) in via Lata, che QP 177 colloca in via Lanza, dove non esiste: trasformazione per rilocazione (D-036). Cap. 4, § 4.2 (r. 45): «la stampa del 1957 colloca in via Lanza – abbinamento privo di riscontro reale per l'edificio […] –, laddove il dattiloscritto registrava correttamente via Lata».</t>
+          <t>Palazzo reale (Simonetti o De Carolis) in via Lata, che QPa 177 colloca in via Lanza, dove non esiste: trasformazione per rilocazione (D-036). Cap. 4, § 4.2 (r. 45): «la stampa del 1957 colloca in via Lanza – abbinamento privo di riscontro reale per l'edificio […] –, laddove il dattiloscritto registrava correttamente via Lata».</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -3129,7 +3129,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Cap. 4, § 4.3 (r. 83): «Robine Vecchie», che entrambe le edizioni conservano a testo (RR II, p. 154; QP 169), «non registrato nelle carte topografiche»: refuso per «Robinie vecchie» o «Rovine vecchie», oppure «ironico abbassamento» delle Rovine della zona; r. 93: situata «tra le Frattocchie e i Due Santi» (ancoraggio relazionale).</t>
+          <t>Cap. 4, § 4.3 (r. 83): «Robine Vecchie», che entrambe le edizioni conservano a testo (RR II, p. 154; QPa 169), «non registrato nelle carte topografiche»: refuso per «Robinie vecchie» o «Rovine vecchie», oppure «ironico abbassamento» delle Rovine della zona; r. 93: situata «tra le Frattocchie e i Due Santi» (ancoraggio relazionale).</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
@@ -4140,7 +4140,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>Due identificazioni concorrenti della «stazione di Castello» (QP 279): Castel Gandolfo (lettura immediata, A-0001) e Castel Savello (Manzotti, A-0002, adottata). Cap. 4, § 4.4 (r. 107).</t>
+          <t>Due identificazioni concorrenti della «stazione di Castello» (QPa 279): Castel Gandolfo (lettura immediata, A-0001) e Castel Savello (Manzotti, A-0002, adottata). Cap. 4, § 4.4 (r. 107).</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -4220,7 +4220,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Quale palazzo reale sta dietro il «palazzo Simonetti» in via Lanza (QP 177): il palazzo Simonetti / De Carolis in via Lata del dattiloscritto (Pinotti) o il palazzo Odescalchi Simonetti di via Vittoria Colonna (Terzoli, cit. ivi). Cap. 4, § 4.2 (r. 45).</t>
+          <t>Quale palazzo reale sta dietro il «palazzo Simonetti» in via Lanza (QPa 177): il palazzo Simonetti / De Carolis in via Lata del dattiloscritto (Pinotti) o il palazzo Odescalchi Simonetti di via Vittoria Colonna (Terzoli, cit. ivi). Cap. 4, § 4.2 (r. 45).</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
@@ -4300,7 +4300,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>«Robine Vecchie» (QP 169) non è registrato nelle carte topografiche: refuso per «Robinie vecchie» o «Rovine vecchie», oppure «ironico abbassamento» delle Rovine della zona; Pinotti conserva la lezione. Cap. 4, § 4.3 (r. 83).</t>
+          <t>«Robine Vecchie» (QPa 169) non è registrato nelle carte topografiche: refuso per «Robinie vecchie» o «Rovine vecchie», oppure «ironico abbassamento» delle Rovine della zona; Pinotti conserva la lezione. Cap. 4, § 4.3 (r. 83).</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
@@ -4450,7 +4450,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>«d'in vetta al crinale degli Ernici o dei Simbruini» (QP 215): identificazione per disgiunzione, non risolta dal testo (WO T-16; Cap. 4, § 4.4).</t>
+          <t>«d'in vetta al crinale degli Ernici o dei Simbruini» (QPa 215): identificazione per disgiunzione, non risolta dal testo (WO T-16; Cap. 4, § 4.4).</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
@@ -4530,7 +4530,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>«Càrsoli» (QP 210) in luogo della grafia corretta Carsòli, «frutto verosimilmente di un'attrazione analogica con la vicina Àrsoli» (Cap. 4, § 4.4, r. 111). Discrepanza di forma registrata, non corretta.</t>
+          <t>«Càrsoli» (QPa 210) in luogo della grafia corretta Carsòli, «frutto verosimilmente di un'attrazione analogica con la vicina Àrsoli» (Cap. 4, § 4.4, r. 111). Discrepanza di forma registrata, non corretta.</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -4692,7 +4692,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>«Gadda sembra infatti proiettare sul personaggio di Ingravallo una propria tessera autobiografica»: la memoria della morte del fratello Enrico e del lutto materno (QP 61, Dosso Faiti).</t>
+          <t>«Gadda sembra infatti proiettare sul personaggio di Ingravallo una propria tessera autobiografica»: la memoria della morte del fratello Enrico e del lutto materno (QPa 61, Dosso Faiti).</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>La «mamma» rinvia al «figlio e fante don Ciccio», e forse ai suoi fratelli caduti in guerra (QP 61, Dosso Faiti).</t>
+          <t>La «mamma» rinvia al «figlio e fante don Ciccio», e forse ai suoi fratelli caduti in guerra (QPa 61, Dosso Faiti).</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
@@ -4839,7 +4839,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>La sequenza «sovrappone la memoria del personaggio, anzi la sovrimprime, a quella dell'autore» (QP 61, Dosso Faiti).</t>
+          <t>La sequenza «sovrappone la memoria del personaggio, anzi la sovrimprime, a quella dell'autore» (QPa 61, Dosso Faiti).</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
@@ -4911,7 +4911,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>«Gadda sembra infatti proiettare sul personaggio di Ingravallo una propria tessera autobiografica»: la memoria della morte del fratello Enrico e del lutto materno (QP 61, Monte Cengio).</t>
+          <t>«Gadda sembra infatti proiettare sul personaggio di Ingravallo una propria tessera autobiografica»: la memoria della morte del fratello Enrico e del lutto materno (QPa 61, Monte Cengio).</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>La «mamma» rinvia al «figlio e fante don Ciccio», e forse ai suoi fratelli caduti in guerra (QP 61, Monte Cengio).</t>
+          <t>La «mamma» rinvia al «figlio e fante don Ciccio», e forse ai suoi fratelli caduti in guerra (QPa 61, Monte Cengio).</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
@@ -5058,7 +5058,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>La sequenza «sovrappone la memoria del personaggio, anzi la sovrimprime, a quella dell'autore» (QP 61, Monte Cengio).</t>
+          <t>La sequenza «sovrappone la memoria del personaggio, anzi la sovrimprime, a quella dell'autore» (QPa 61, Monte Cengio).</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
@@ -5259,7 +5259,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>Lettura del censimento: palazzo reale, ancorato a via Lanza dove lo pone QP 177.</t>
+          <t>Lettura del censimento: palazzo reale, ancorato a via Lanza dove lo pone QPa 177.</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
@@ -5445,7 +5445,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>qp</t>
+          <t>qpa</t>
         </is>
       </c>
       <c r="H74" t="n">
@@ -5453,7 +5453,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>Fattocchie (RR II 219, stampa Garzanti) / Frattocchie (QP 241): emendamento dell'editore. Le occorrenze si annotano sulla lezione del testo di riferimento.</t>
+          <t>Fattocchie (QP, RR II 219) / Frattocchie (QPa 241): emendamento dell'editore.</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
@@ -5518,7 +5518,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>via Lata (dtsFG) / via Lanza (QP 177): il dattiloscritto dei capitoli nuovi colloca il palazzo Simonetti nella via reale in cui si trova; la stampa lo sposta in via Lanza, dove non esiste (D-036).</t>
+          <t>via Lata (dtsFG) / via Lanza (QPa 177): il dattiloscritto dei capitoli nuovi colloca il palazzo Simonetti nella via reale in cui si trova; la stampa lo sposta in via Lanza, dove non esiste (D-036).</t>
         </is>
       </c>
       <c r="L75" t="inlineStr">
@@ -5585,7 +5585,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>Civico 119 (QPL 285) / 219 (QP 16).</t>
+          <t>Civico 119 (QPL 285) / 219 (QPa 16).</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
@@ -5595,7 +5595,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>Corrispondenza QPL 285 ↔ QP 16 confermata da LS (9/10/2026). Cap. 4, § 4.2 (r. 45).</t>
+          <t>Corrispondenza QPL 285 ↔ QPa 16 confermata da LS (9/10/2026). Cap. 4, § 4.2 (r. 45).</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
@@ -5652,7 +5652,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>Civico 119 (QPL 293) / 219 (QP 25).</t>
+          <t>Civico 119 (QPL 293) / 219 (QPa 25).</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
@@ -5662,7 +5662,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>Corrispondenza QPL 293 ↔ QP 25 confermata da LS (9/10/2026). Cap. 4, § 4.2 (r. 45).</t>
+          <t>Corrispondenza QPL 293 ↔ QPa 25 confermata da LS (9/10/2026). Cap. 4, § 4.2 (r. 45).</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
@@ -5719,7 +5719,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>«palazzo degli ori» (QPL 285) / «palazzo dell'Oro» (QP 16).</t>
+          <t>«palazzo degli ori» (QPL 285) / «palazzo dell'Oro» (QPa 16).</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
@@ -5729,7 +5729,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>Corrispondenza QPL 285 ↔ QP 16 confermata da LS (9/10/2026). Cap. 4, § 4.2 (r. 45).</t>
+          <t>Corrispondenza QPL 285 ↔ QPa 16 confermata da LS (9/10/2026). Cap. 4, § 4.2 (r. 45).</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -5786,7 +5786,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>«palazzo degli ori» (QPL 293) / «palazzo dell'Oro» (QP 25).</t>
+          <t>«palazzo degli ori» (QPL 293) / «palazzo dell'Oro» (QPa 25).</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
@@ -5796,7 +5796,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>Corrispondenza QPL 293 ↔ QP 25 confermata da LS (9/10/2026). Cap. 4, § 4.2 (r. 45).</t>
+          <t>Corrispondenza QPL 293 ↔ QPa 25 confermata da LS (9/10/2026). Cap. 4, § 4.2 (r. 45).</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>qp</t>
+          <t>qpa</t>
         </is>
       </c>
       <c r="H80" t="n">
@@ -5913,7 +5913,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>qp</t>
+          <t>qpa</t>
         </is>
       </c>
       <c r="H81" t="n">
@@ -5936,7 +5936,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>Separato dal tragitto di QP 297 (D-060). È un elenco disgiuntivo e abituale di provenienze, non una sequenza: potrebbe non essere un percorso.</t>
+          <t>Separato dal tragitto di QPa 297 (D-060). È un elenco disgiuntivo e abituale di provenienze, non una sequenza: potrebbe non essere un percorso.</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -5983,7 +5983,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>qp</t>
+          <t>qpa</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -6050,7 +6050,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>qp</t>
+          <t>qpa</t>
         </is>
       </c>
       <c r="H83" t="n">
@@ -6120,7 +6120,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>qp</t>
+          <t>qpa</t>
         </is>
       </c>
       <c r="H84" t="n">
@@ -6185,7 +6185,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>qp</t>
+          <t>qpa</t>
         </is>
       </c>
       <c r="H85" t="n">
@@ -6198,7 +6198,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>«La strada era una sola, pe fortuna, salvo il primo pezzo però: la statale, l'Appia, poi ad angolo retto la deviazione della provinciale, pe Falcognana»: la strada spiegata dopo le indicazioni di Camilla (QP 237).</t>
+          <t>«La strada era una sola, pe fortuna, salvo il primo pezzo però: la statale, l'Appia, poi ad angolo retto la deviazione della provinciale, pe Falcognana»: la strada spiegata dopo le indicazioni di Camilla (QPa 237).</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
@@ -6255,7 +6255,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>qp</t>
+          <t>qpa</t>
         </is>
       </c>
       <c r="H86" t="n">
@@ -6325,7 +6325,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>qp</t>
+          <t>qpa</t>
         </is>
       </c>
       <c r="H87" t="n">
@@ -6395,7 +6395,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>qp</t>
+          <t>qpa</t>
         </is>
       </c>
       <c r="H88" t="n">
@@ -6465,7 +6465,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>qp</t>
+          <t>qpa</t>
         </is>
       </c>
       <c r="H89" t="n">
@@ -6488,7 +6488,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>Come QP 169: elenco disgiuntivo e abituale, non una sequenza.</t>
+          <t>Come QPa 169: elenco disgiuntivo e abituale, non una sequenza.</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -6535,7 +6535,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>qp</t>
+          <t>qpa</t>
         </is>
       </c>
       <c r="H90" t="n">
@@ -6605,7 +6605,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>qp</t>
+          <t>qpa</t>
         </is>
       </c>
       <c r="H91" t="n">
@@ -6675,7 +6675,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>qp</t>
+          <t>qpa</t>
         </is>
       </c>
       <c r="H92" t="n">
@@ -6745,7 +6745,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>qp</t>
+          <t>qpa</t>
         </is>
       </c>
       <c r="H93" t="n">
@@ -6810,7 +6810,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>qp</t>
+          <t>qpa</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -6877,7 +6877,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>qp</t>
+          <t>qpa</t>
         </is>
       </c>
       <c r="H95" t="n">
@@ -6947,7 +6947,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>qp</t>
+          <t>qpa</t>
         </is>
       </c>
       <c r="H96" t="n">
@@ -7012,7 +7012,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>qp</t>
+          <t>qpa</t>
         </is>
       </c>
       <c r="H97" t="n">
@@ -7082,7 +7082,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>qp</t>
+          <t>qpa</t>
         </is>
       </c>
       <c r="H98" t="n">
@@ -7152,7 +7152,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>qp</t>
+          <t>qpa</t>
         </is>
       </c>
       <c r="H99" t="n">
@@ -7222,7 +7222,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>qp</t>
+          <t>qpa</t>
         </is>
       </c>
       <c r="H100" t="n">
@@ -7446,7 +7446,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>Luogo: via_delle_oche (QP 22). Soggetto l'entità dell'ancora, per la regola dell'asse geometria (D-070); lo statuto del luogo non cambia (D-072).</t>
+          <t>Luogo: via_delle_oche (QPa 22). Soggetto l'entità dell'ancora, per la regola dell'asse geometria (D-070); lo statuto del luogo non cambia (D-072).</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">

</xml_diff>

<commit_message>
chiusura delle voci aperte della fase 2: motivazioni, Violation, estratti (D-078…D-083)
48 motivazioni di statuto validate (33 così come sono, 5 riscritte, 10
nuove); StatusRationaleShape a Violation, SHACL senza risultati; estratti
delle occorrenze divise verificati; nuove fonti Terzoli 2008 e Guida TCI
1925. Restano aperti Cassero, carta TCI di Manzotti, Nota al testo di
Pinotti 2018, identificatori esterni, data del Censimento (non fornita).
ABox 40.472 -> 40.507.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Assertions.xlsx
+++ b/data/source/xlsx/Assertions.xlsx
@@ -713,7 +713,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -780,7 +780,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>annotator/lorenzo_sabatino</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Nessuna motivazione nei documenti del progetto (descrizione vuota, nessun passo del Cap. 4): da compilare.</t>
+          <t>Bottega senza riscontro nei repertori: nome e collocazione d'autore.</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -842,12 +842,17 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione nuova di LS (10/10/2026, D-080).</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -874,7 +879,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>annotator/lorenzo_sabatino</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -889,7 +894,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Nessuna motivazione nei documenti del progetto (descrizione vuota, nessun passo del Cap. 4): da compilare.</t>
+          <t>Denominazione popolare di un luogo reale presso Sant'Ignazio a Roma: il Buco a Sant'Ignazio (ancora gaz_buco_a_santignazio, 41,898 N 12,480 E).</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -899,12 +904,17 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione nuova di LS (10/10/2026, D-080).</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -939,6 +949,14 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>512</v>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
           <t>si</t>
@@ -946,7 +964,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Nessuna motivazione nei documenti del progetto (descrizione vuota, nessun passo del Cap. 4): da compilare.</t>
+          <t>Località reale nei pressi della stazione delle Frattocchie.</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -956,12 +974,17 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione nuova di LS (10/10/2026, D-080).</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1041,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1028,7 +1051,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1085,7 +1108,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1095,7 +1118,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1175,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1162,7 +1185,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1242,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1229,7 +1252,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1381,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1368,7 +1391,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1418,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>annotator/lorenzo_sabatino</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1403,6 +1426,14 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>qpa</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>169</v>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
           <t>si</t>
@@ -1410,7 +1441,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Nessuna motivazione nei documenti del progetto (descrizione vuota, nessun passo del Cap. 4): da compilare.</t>
+          <t>Toponimo senza riscontro, collocato dal testo "a Sant'Ignazio", fra le provenienze di QPa 169.</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1420,12 +1451,17 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione nuova di LS (10/10/2026, D-080).</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1477,7 +1513,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Cap. 4, § 4.3 (r. 85): la denominazione è una «deformazione paraetimologica d'un toponimo reale» (Castelporziano, «il che penderebbe verso il luogo trasformato»), mentre la festa notturna «appartiene a uno spazio onirico e destrutturato, privo di collocazione metrica e dunque ascrivibile alla categoria dell'immaginato». Perimetro d'identità da dichiarare (H3, DC-09, DC-11).</t>
+          <t>Luogo senza corrispondenza con un luogo attestato: il nome deforma Castelporziano, ma la festa notturna appartiene a uno spazio d'immaginazione d'autore.</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1487,7 +1523,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione riscritta da LS (10/10/2026, D-079).</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1497,7 +1533,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1635,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>annotator/lorenzo_sabatino</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1614,7 +1650,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Nessuna motivazione nei documenti del progetto (descrizione vuota, nessun passo del Cap. 4): da compilare.</t>
+          <t>Luogo del mondo diegetico della Zamira: segue lo statuto del laboratorio (laboratorio_zamira).</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1624,12 +1660,17 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione nuova di LS (10/10/2026, D-080).</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1686,7 +1727,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1696,7 +1737,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1723,7 +1764,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>annotator/lorenzo_sabatino</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1738,7 +1779,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Nessuna motivazione nei documenti del progetto (descrizione vuota, nessun passo del Cap. 4): da compilare.</t>
+          <t>Perifrasi d'autore per colli reali: i Colli Albani (ancora gaz_colli_albani).</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -1748,12 +1789,17 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione nuova di LS (10/10/2026, D-080).</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1788,6 +1834,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
           <t>si</t>
@@ -1795,7 +1846,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Nessuna motivazione nei documenti del progetto (descrizione vuota, nessun passo del Cap. 4): da compilare.</t>
+          <t>Terzoli ricostruisce l'origine onomastica di Ciurlani e il gioco di parole con "truffaldino"; nessun elemento di collocazione topografica.</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -1805,12 +1856,17 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione nuova di LS (10/10/2026, D-080). Pagina di Terzoli 2015 da compilare.</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1998,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -1952,7 +2008,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2009,7 +2065,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2019,7 +2075,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2076,7 +2132,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2086,7 +2142,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2143,7 +2199,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2153,7 +2209,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2210,7 +2266,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2220,7 +2276,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2247,7 +2303,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>annotator/lorenzo_sabatino</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2257,8 +2313,11 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>sabatino_cap4</t>
-        </is>
+          <t>qpa</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>173</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -2267,7 +2326,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Cap. 4, § 4.3 (r. 85): «il Monte Nuncupale, posto a chiusura d'un orizzonte che spazia «da Rocca di Papa a Castel Savelli, giù: da Rocca Orsina al Monte Nuncupale, su» (QP 173)», fra i luoghi inventati. NB: nei dati è Imagined dopo la permutazione (D-030, D-035).</t>
+          <t>Monte senza corrispondenza con un rilievo attestato; l'autore lo immagina a chiusura dell'orizzonte dei Colli Albani ("da Rocca Orsina al Monte Nuncupale, su", QPa 173).</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -2277,7 +2336,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione riscritta da LS (10/10/2026, D-079).</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2287,7 +2346,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2344,7 +2403,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2354,7 +2413,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2411,7 +2470,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2421,7 +2480,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2448,7 +2507,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>annotator/lorenzo_sabatino</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2463,7 +2522,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Nessuna motivazione nei documenti del progetto (descrizione vuota, nessun passo del Cap. 4): da compilare.</t>
+          <t>Palazzo Venezia, sede di Mussolini, indicato per antonomasia dalla Sala del Mappamondo e deformato in "Mappamonno": referente reale, nome trasformato.</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -2473,12 +2532,17 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione nuova di LS (10/10/2026, D-080).</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2543,7 +2607,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2553,7 +2617,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2610,7 +2674,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2620,7 +2684,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2677,7 +2741,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2687,7 +2751,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2744,7 +2808,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -2754,7 +2818,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2811,7 +2875,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -2821,7 +2885,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2856,6 +2920,16 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>911 (cfr. Terzoli 2008, pp. 109–113)</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr">
         <is>
           <t>si</t>
@@ -2863,7 +2937,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Nessuna motivazione nei documenti del progetto (descrizione vuota, nessun passo del Cap. 4): da compilare.</t>
+          <t>Strada che dall'Anziate va verso Casal Bruciato, parallela alla strada di Falconara percorsa da Pestalozzi, e scavalca la ferrovia Roma–Velletri in località Ponte di Santa Fumia: planimetria e toponimi corrispondono a quelli delle cartine della Guida Touring 1925 (tra le pp. 736–737, cart. 4, e 758–759, cart. 1).</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -2873,12 +2947,17 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione nuova di LS (10/10/2026, D-080).</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2935,7 +3014,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2945,7 +3024,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3002,7 +3081,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -3012,7 +3091,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3069,7 +3148,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3079,7 +3158,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3218,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3149,7 +3228,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3176,7 +3255,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>annotator/lorenzo_sabatino</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -3186,8 +3265,11 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>sabatino_cap4</t>
-        </is>
+          <t>qpa</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>107</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
@@ -3196,7 +3278,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Cap. 4, § 4.3 (r. 85): tra i luoghi inventati con «una precisa collocazione topografica», «Roccafringoli, situata «su su in cima ai monti, a monte Manno, quasi, che da Palestrina ce se va cor ciuccio» (QP 107)». NB: il capitolo lo dice inventato; nei dati è Imagined dopo la permutazione (D-030, D-035).</t>
+          <t>Paese senza corrispondenza con un luogo attestato; l'autore lo immagina sui monti presso Palestrina ("a monte Manno, quasi", QPa 107).</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -3206,7 +3288,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione riscritta da LS (10/10/2026, D-079).</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3216,7 +3298,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3273,7 +3355,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3283,7 +3365,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3340,7 +3422,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3350,7 +3432,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3407,7 +3489,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3417,7 +3499,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3444,7 +3526,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>annotator/lorenzo_sabatino</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -3454,8 +3536,11 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>sabatino_cap4</t>
-        </is>
+          <t>qpa</t>
+        </is>
+      </c>
+      <c r="H46" t="n">
+        <v>141</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
@@ -3464,7 +3549,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Cap. 4, § 4.3 (r. 85): «Scerpure, la favolosa città del maharajah posizionata «sulle rive, più o meno, del nativo Brahmaputra» (QP 141)», fra i luoghi inventati; «Scerpure esibisce un nome inventato a fronte d'una collocazione geografica nota». NB: nei dati è Imagined dopo la permutazione (D-030, D-035).</t>
+          <t>Città senza corrispondenza con un luogo attestato; l'autore la immagina "sulle rive, più o meno, del nativo Brahmaputra" (QPa 141).</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -3474,7 +3559,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione riscritta da LS (10/10/2026, D-079).</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3484,7 +3569,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3541,7 +3626,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3551,7 +3636,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3608,7 +3693,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3618,7 +3703,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3675,7 +3760,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3685,7 +3770,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3747,7 +3832,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3757,7 +3842,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3814,7 +3899,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3824,7 +3909,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3969,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -3894,7 +3979,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3921,7 +4006,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>annotator/lorenzo_sabatino</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -3931,8 +4016,11 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>censimento_gaddatlas</t>
-        </is>
+          <t>qpa</t>
+        </is>
+      </c>
+      <c r="H53" t="n">
+        <v>22</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
@@ -3941,7 +4029,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Descrizione del censimento: «via topograficamente non precisata».</t>
+          <t>Via reale di Bologna, nota via di prostituzione, che il testo traslata a Milano (QPa 22; U-0009).</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -3951,7 +4039,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione riscritta da LS (10/10/2026, D-079).</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -3961,7 +4049,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3988,7 +4076,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>annotator/lorenzo_sabatino</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -4003,7 +4091,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Nessuna motivazione nei documenti del progetto (descrizione vuota, nessun passo del Cap. 4): da compilare.</t>
+          <t>Villino senza riscontro, collocato dal testo sul Lungotevere.</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -4013,12 +4101,17 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione nuova di LS (10/10/2026, D-080).</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Chiusura delle voci aperte della fase 2 (D-078…D-083) (#3)
48 motivazioni di statuto validate (33 così come sono, 5 riscritte, 10
nuove); StatusRationaleShape a Violation, SHACL senza risultati; estratti
delle occorrenze divise verificati; nuove fonti Terzoli 2008 e Guida TCI
1925. Restano aperti Cassero, carta TCI di Manzotti, Nota al testo di
Pinotti 2018, identificatori esterni, data del Censimento (non fornita).
ABox 40.472 -> 40.507.

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Assertions.xlsx
+++ b/data/source/xlsx/Assertions.xlsx
@@ -713,7 +713,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -780,7 +780,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>annotator/lorenzo_sabatino</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Nessuna motivazione nei documenti del progetto (descrizione vuota, nessun passo del Cap. 4): da compilare.</t>
+          <t>Bottega senza riscontro nei repertori: nome e collocazione d'autore.</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -842,12 +842,17 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione nuova di LS (10/10/2026, D-080).</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -874,7 +879,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>annotator/lorenzo_sabatino</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -889,7 +894,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Nessuna motivazione nei documenti del progetto (descrizione vuota, nessun passo del Cap. 4): da compilare.</t>
+          <t>Denominazione popolare di un luogo reale presso Sant'Ignazio a Roma: il Buco a Sant'Ignazio (ancora gaz_buco_a_santignazio, 41,898 N 12,480 E).</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -899,12 +904,17 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione nuova di LS (10/10/2026, D-080).</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -939,6 +949,14 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>512</v>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
           <t>si</t>
@@ -946,7 +964,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Nessuna motivazione nei documenti del progetto (descrizione vuota, nessun passo del Cap. 4): da compilare.</t>
+          <t>Località reale nei pressi della stazione delle Frattocchie.</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -956,12 +974,17 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione nuova di LS (10/10/2026, D-080).</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1041,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1028,7 +1051,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1085,7 +1108,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1095,7 +1118,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1175,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1162,7 +1185,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1242,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1229,7 +1252,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1381,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1368,7 +1391,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1418,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>annotator/lorenzo_sabatino</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1403,6 +1426,14 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>qpa</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>169</v>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
           <t>si</t>
@@ -1410,7 +1441,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Nessuna motivazione nei documenti del progetto (descrizione vuota, nessun passo del Cap. 4): da compilare.</t>
+          <t>Toponimo senza riscontro, collocato dal testo "a Sant'Ignazio", fra le provenienze di QPa 169.</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1420,12 +1451,17 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione nuova di LS (10/10/2026, D-080).</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1477,7 +1513,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Cap. 4, § 4.3 (r. 85): la denominazione è una «deformazione paraetimologica d'un toponimo reale» (Castelporziano, «il che penderebbe verso il luogo trasformato»), mentre la festa notturna «appartiene a uno spazio onirico e destrutturato, privo di collocazione metrica e dunque ascrivibile alla categoria dell'immaginato». Perimetro d'identità da dichiarare (H3, DC-09, DC-11).</t>
+          <t>Luogo senza corrispondenza con un luogo attestato: il nome deforma Castelporziano, ma la festa notturna appartiene a uno spazio d'immaginazione d'autore.</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1487,7 +1523,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione riscritta da LS (10/10/2026, D-079).</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1497,7 +1533,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1635,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>annotator/lorenzo_sabatino</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1614,7 +1650,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Nessuna motivazione nei documenti del progetto (descrizione vuota, nessun passo del Cap. 4): da compilare.</t>
+          <t>Luogo del mondo diegetico della Zamira: segue lo statuto del laboratorio (laboratorio_zamira).</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1624,12 +1660,17 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione nuova di LS (10/10/2026, D-080).</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1686,7 +1727,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1696,7 +1737,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1723,7 +1764,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>annotator/lorenzo_sabatino</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1738,7 +1779,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Nessuna motivazione nei documenti del progetto (descrizione vuota, nessun passo del Cap. 4): da compilare.</t>
+          <t>Perifrasi d'autore per colli reali: i Colli Albani (ancora gaz_colli_albani).</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -1748,12 +1789,17 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione nuova di LS (10/10/2026, D-080).</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1788,6 +1834,11 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
           <t>si</t>
@@ -1795,7 +1846,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Nessuna motivazione nei documenti del progetto (descrizione vuota, nessun passo del Cap. 4): da compilare.</t>
+          <t>Terzoli ricostruisce l'origine onomastica di Ciurlani e il gioco di parole con "truffaldino"; nessun elemento di collocazione topografica.</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -1805,12 +1856,17 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione nuova di LS (10/10/2026, D-080). Pagina di Terzoli 2015 da compilare.</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1998,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -1952,7 +2008,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2009,7 +2065,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2019,7 +2075,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2076,7 +2132,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2086,7 +2142,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2143,7 +2199,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2153,7 +2209,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2210,7 +2266,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2220,7 +2276,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2247,7 +2303,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>annotator/lorenzo_sabatino</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2257,8 +2313,11 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>sabatino_cap4</t>
-        </is>
+          <t>qpa</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>173</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -2267,7 +2326,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Cap. 4, § 4.3 (r. 85): «il Monte Nuncupale, posto a chiusura d'un orizzonte che spazia «da Rocca di Papa a Castel Savelli, giù: da Rocca Orsina al Monte Nuncupale, su» (QP 173)», fra i luoghi inventati. NB: nei dati è Imagined dopo la permutazione (D-030, D-035).</t>
+          <t>Monte senza corrispondenza con un rilievo attestato; l'autore lo immagina a chiusura dell'orizzonte dei Colli Albani ("da Rocca Orsina al Monte Nuncupale, su", QPa 173).</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -2277,7 +2336,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione riscritta da LS (10/10/2026, D-079).</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2287,7 +2346,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2344,7 +2403,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2354,7 +2413,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2411,7 +2470,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2421,7 +2480,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2448,7 +2507,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>annotator/lorenzo_sabatino</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2463,7 +2522,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Nessuna motivazione nei documenti del progetto (descrizione vuota, nessun passo del Cap. 4): da compilare.</t>
+          <t>Palazzo Venezia, sede di Mussolini, indicato per antonomasia dalla Sala del Mappamondo e deformato in "Mappamonno": referente reale, nome trasformato.</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -2473,12 +2532,17 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione nuova di LS (10/10/2026, D-080).</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2543,7 +2607,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2553,7 +2617,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2610,7 +2674,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2620,7 +2684,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2677,7 +2741,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2687,7 +2751,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2744,7 +2808,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -2754,7 +2818,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2811,7 +2875,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -2821,7 +2885,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2856,6 +2920,16 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>911 (cfr. Terzoli 2008, pp. 109–113)</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr">
         <is>
           <t>si</t>
@@ -2863,7 +2937,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Nessuna motivazione nei documenti del progetto (descrizione vuota, nessun passo del Cap. 4): da compilare.</t>
+          <t>Strada che dall'Anziate va verso Casal Bruciato, parallela alla strada di Falconara percorsa da Pestalozzi, e scavalca la ferrovia Roma–Velletri in località Ponte di Santa Fumia: planimetria e toponimi corrispondono a quelli delle cartine della Guida Touring 1925 (tra le pp. 736–737, cart. 4, e 758–759, cart. 1).</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -2873,12 +2947,17 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione nuova di LS (10/10/2026, D-080).</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -2935,7 +3014,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2945,7 +3024,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3002,7 +3081,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -3012,7 +3091,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3069,7 +3148,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3079,7 +3158,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3218,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3149,7 +3228,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3176,7 +3255,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>annotator/lorenzo_sabatino</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -3186,8 +3265,11 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>sabatino_cap4</t>
-        </is>
+          <t>qpa</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>107</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
@@ -3196,7 +3278,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Cap. 4, § 4.3 (r. 85): tra i luoghi inventati con «una precisa collocazione topografica», «Roccafringoli, situata «su su in cima ai monti, a monte Manno, quasi, che da Palestrina ce se va cor ciuccio» (QP 107)». NB: il capitolo lo dice inventato; nei dati è Imagined dopo la permutazione (D-030, D-035).</t>
+          <t>Paese senza corrispondenza con un luogo attestato; l'autore lo immagina sui monti presso Palestrina ("a monte Manno, quasi", QPa 107).</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -3206,7 +3288,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione riscritta da LS (10/10/2026, D-079).</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3216,7 +3298,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3273,7 +3355,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3283,7 +3365,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3340,7 +3422,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3350,7 +3432,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3407,7 +3489,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3417,7 +3499,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3444,7 +3526,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>annotator/lorenzo_sabatino</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -3454,8 +3536,11 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>sabatino_cap4</t>
-        </is>
+          <t>qpa</t>
+        </is>
+      </c>
+      <c r="H46" t="n">
+        <v>141</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
@@ -3464,7 +3549,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Cap. 4, § 4.3 (r. 85): «Scerpure, la favolosa città del maharajah posizionata «sulle rive, più o meno, del nativo Brahmaputra» (QP 141)», fra i luoghi inventati; «Scerpure esibisce un nome inventato a fronte d'una collocazione geografica nota». NB: nei dati è Imagined dopo la permutazione (D-030, D-035).</t>
+          <t>Città senza corrispondenza con un luogo attestato; l'autore la immagina "sulle rive, più o meno, del nativo Brahmaputra" (QPa 141).</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -3474,7 +3559,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione riscritta da LS (10/10/2026, D-079).</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3484,7 +3569,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3541,7 +3626,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3551,7 +3636,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3608,7 +3693,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3618,7 +3703,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3675,7 +3760,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3685,7 +3770,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3747,7 +3832,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3757,7 +3842,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3814,7 +3899,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3824,7 +3909,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3969,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Validata da LS (10/10/2026, D-078).</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -3894,7 +3979,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3921,7 +4006,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>annotator/lorenzo_sabatino</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -3931,8 +4016,11 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>censimento_gaddatlas</t>
-        </is>
+          <t>qpa</t>
+        </is>
+      </c>
+      <c r="H53" t="n">
+        <v>22</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
@@ -3941,7 +4029,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Descrizione del censimento: «via topograficamente non precisata».</t>
+          <t>Via reale di Bologna, nota via di prostituzione, che il testo traslata a Milano (QPa 22; U-0009).</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -3951,7 +4039,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione riscritta da LS (10/10/2026, D-079).</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -3961,7 +4049,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>
@@ -3988,7 +4076,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>annotator/lorenzo_sabatino</t>
+          <t>lorenzo_sabatino</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -4003,7 +4091,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Nessuna motivazione nei documenti del progetto (descrizione vuota, nessun passo del Cap. 4): da compilare.</t>
+          <t>Villino senza riscontro, collocato dal testo sul Lungotevere.</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -4013,12 +4101,17 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>Bozza T-33 (D-046): da validare in REVIEW_2</t>
+          <t>Motivazione nuova di LS (10/10/2026, D-080).</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>bozza</t>
+          <t>validata</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tre tipi di lettura per i loci critici; varianti di forma e di sostituzione (blocco A, D-085)
RepertoryAttestation, NamingAssertion (NamingMechanismScheme, playsOn),
CommentaryAssertion; chora:quotation sull'atto; variantKind (FormVariant,
SubstitutionVariant); cito:disagreesWith. Shape 24.
TBox 1.473 -> 1.612.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Assertions.xlsx
+++ b/data/source/xlsx/Assertions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S103"/>
+  <dimension ref="A1:W103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -512,6 +512,26 @@
           <t>Original_Source</t>
         </is>
       </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Quotation</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Plays_On</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Variant_Kind</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Disagrees_With</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -5569,6 +5589,11 @@
           <t>validata</t>
         </is>
       </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>forma</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5634,6 +5659,11 @@
           <t>validata</t>
         </is>
       </c>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t>forma</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5701,6 +5731,11 @@
           <t>validata</t>
         </is>
       </c>
+      <c r="V76" t="inlineStr">
+        <is>
+          <t>forma</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5768,6 +5803,11 @@
           <t>validata</t>
         </is>
       </c>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>forma</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -5835,6 +5875,11 @@
           <t>validata</t>
         </is>
       </c>
+      <c r="V78" t="inlineStr">
+        <is>
+          <t>forma</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -5900,6 +5945,11 @@
       <c r="O79" t="inlineStr">
         <is>
           <t>validata</t>
+        </is>
+      </c>
+      <c r="V79" t="inlineStr">
+        <is>
+          <t>forma</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
loci critici: 56 letture, osteriuccia del bivio, Cassero, varianti di sostituzione (blocco C, D-087)
Attestazioni nel repertorio (25), identificazioni (11), commenti (10),
letture onomastiche (6), varianti di sostituzione (2), incertezza (1),
statuto dell'osteriuccia. Nuovo luogo osteriuccia_bivio (QPa 239) in
carta; Cassero in un'interpretazione: IQ20 = 0 e Violation. Quattro entità
senza coordinate. Statuti generati citano le attestazioni.
ABox 40.553 -> 42.501; feature 301 -> 302.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Assertions.xlsx
+++ b/data/source/xlsx/Assertions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W103"/>
+  <dimension ref="A1:W159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1859,6 +1859,11 @@
           <t>terzoli_2015</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>433–435, 644</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
           <t>si</t>
@@ -1876,7 +1881,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Motivazione nuova di LS (10/10/2026, D-080). Pagina di Terzoli 2015 da compilare.</t>
+          <t>Validata da LS; pagine di Terzoli 2015 compilate (D-087).</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2535,6 +2540,14 @@
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>537</v>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>si</t>
@@ -3817,14 +3830,14 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
+          <t>manzotti</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
           <t>annotator/lorenzo_sabatino</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>annotator/lorenzo_sabatino</t>
-        </is>
-      </c>
       <c r="G50" t="inlineStr">
         <is>
           <t>manzotti_2010</t>
@@ -3832,7 +3845,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>239, 293</t>
+          <t>293–294</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3852,7 +3865,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>Validata da LS (10/10/2026, D-078).</t>
+          <t>Autore della lettura Manzotti, codificatore LS (D-087).</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -7318,7 +7331,7 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>Nuovo percorso (D-060). La lettura di Manzotti di «per fil a dest» (2010, p. 269) è una nota attribuita di fase 3.</t>
+          <t>Nuovo percorso (D-060). La lettura di Manzotti di «per fil a dest» è K-0008 (D-087).</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
@@ -7615,6 +7628,3968 @@
       <c r="R103" t="inlineStr">
         <is>
           <t>ref_00028</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>N-0001</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>naming</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>reference/ref_00403</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>chora:TypoHypothesis</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>491–492</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>Prima ipotesi di Terzoli: refuso per «Robinie vecchie».</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>ref_00403</t>
+        </is>
+      </c>
+      <c r="T104" t="inlineStr">
+        <is>
+          <t>refuso per «Robinie vecchie»</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>N-0002</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>naming</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>reference/ref_00403</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>chora:TypoHypothesis</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>491–492</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>Seconda ipotesi: refuso per «Rovine vecchie», dai ruderi della zona (Rovina del Pecoraro, della Strega, del Fenilone, presso la Cecchignola).</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="R105" t="inlineStr">
+        <is>
+          <t>ref_00403</t>
+        </is>
+      </c>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t>refuso per «Rovine vecchie»</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>N-0003</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>naming</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>reference/ref_00403</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>chora:IronicLowering</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>491–492</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>Terza ipotesi: «ironico abbassamento» delle «rovine» della zona, per parafrasi e paronomasia.</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="R106" t="inlineStr">
+        <is>
+          <t>ref_00403</t>
+        </is>
+      </c>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t>«ironico abbassamento»</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>K-0001</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>commentary</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>reference/ref_00403</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>italia</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>italia_2020</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>102–103</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Secondo Italia, Pinotti 2018 emenda «Robine» come refuso di Garzanti 1992.</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="R107" t="inlineStr">
+        <is>
+          <t>ref_00403</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>K-0002</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>commentary</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>reference/ref_00403</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>qpa</t>
+        </is>
+      </c>
+      <c r="H108" t="n">
+        <v>169</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>In Pinotti 2018 non c'è emendamento di «Robine»: QPa 169 legge «Robine Vecchie».</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>Risponde a K-0001 (D-087).</t>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="R108" t="inlineStr">
+        <is>
+          <t>ref_00403</t>
+        </is>
+      </c>
+      <c r="W108" t="inlineStr">
+        <is>
+          <t>K-0001</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>U-0010</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>uncertainty</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>reference/ref_00404</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>chora:Incompleteness</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H109" t="n">
+        <v>492</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>«Cassero» e «Sant'Ignazio»: toponimi che Terzoli non trova nelle carte topografiche.</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="Q109" t="inlineStr">
+        <is>
+          <t>documentaria</t>
+        </is>
+      </c>
+      <c r="R109" t="inlineStr">
+        <is>
+          <t>ref_00404</t>
+        </is>
+      </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>«toponimi non segnalati nelle carte topografiche»</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>K-0003</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>commentary</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>reference/ref_00588</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>italia</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>italia_2020</t>
+        </is>
+      </c>
+      <c r="H110" t="n">
+        <v>101</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>Nessun elemento fa pensare a un'invenzione gaddiana: l'emendamento «Frattocchie» di Pinotti 2018 è giustificato. Concorde con V-0001.</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="R110" t="inlineStr">
+        <is>
+          <t>ref_00588</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>V-0005</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>variant</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>reference/ref_00132</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>reference/ref_00734</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H111" t="n">
+        <v>142</v>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Nel cap. II le fermate del tram («Ai Due Santi, al Torraccio, a le Frattocchie») sostituiscono la sola «Marino» di QPL (RR II, p. 324).</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="R111" t="inlineStr">
+        <is>
+          <t>ref_00132</t>
+        </is>
+      </c>
+      <c r="V111" t="inlineStr">
+        <is>
+          <t>sostituzione</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>I-0001</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>identification</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>narrativeplace/ca_francesi</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_ca_francesi</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H112" t="n">
+        <v>512</v>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>Ca' Francesi: località nei pressi della stazione delle Frattocchie.</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t>«località nei pressi della stazione delle Frattocchie»</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>I-0002</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>identification</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>narrativeplace/tor_ser_paolo</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_tor_ser_paolo</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H113" t="n">
+        <v>512</v>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>Tor ser Paolo, o Torre Messer Paoli, tra via Cavona e via dei Laghi, presso Marino.</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="T113" t="inlineStr">
+        <is>
+          <t>«o Torre Messer Paoli, tra via Cavona e via dei Laghi, presso Marino»</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>I-0003</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>identification</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>narrativeplace/fontana_di_papa</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_fontana_di_papa</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H114" t="n">
+        <v>658</v>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>«La fontana» è Fontana di Papa, frazione di Ariccia, una decina di km a sud delle Frattocchie lungo l'Anziatina (Guida 1924, p. 561).</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="R114" t="inlineStr">
+        <is>
+          <t>ref_00529</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>T-0021</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_fontana_di_papa</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1924</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>658 (Bertarelli 1924, p. 561)</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>Fontana di Papa è registrata nella Guida 1924, p. 561.</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>I-0004</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>identification</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>narrativeplace/osteriuccia_bivio</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_osteria_bivio_frattocchie</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H116" t="n">
+        <v>776</v>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>L'«osteriuccia del bivio» è l'«Osteria» registrata dalla guida sul bivio fra Appia Antica e strada del Divino Amore, presso le Frattocchie. Non adottata: il luogo si posiziona dalle ancore.</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="R116" t="inlineStr">
+        <is>
+          <t>ref_00736</t>
+        </is>
+      </c>
+      <c r="T116" t="inlineStr">
+        <is>
+          <t>«nei pressi delle Frattocchie […] proprio su un bivio tra l'Appia Antica e la strada per il santuario del Divino Amore, è registrata un'"Osteria"»</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>T-0022</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_osteria_bivio_frattocchie</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1925</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>776 (Bertarelli 1925, cart. 1, tra pp. 758–759, «Osteria»; cart. 4, tra pp. 736–737, «Ost.»)</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>L'osteria del bivio è registrata sulle cart. 1 e 4 della Guida 1925.</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>T-0001</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_ciampino</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1925</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>418–419 (Bertarelli 1925, cart. 4, tra pp. 736–737)</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>«Ciampino» è registrato sulla cart. 4 della Guida 1925 (topografia della guida in QP).</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>T-0002</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_tor_ser_paolo</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1925</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>418–419 (Bertarelli 1925, cart. 4, tra pp. 736–737)</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>«Tor ser Paolo» è registrato sulla cart. 4 della Guida 1925 (topografia della guida in QP).</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N119" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>T-0003</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_frattocchie</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1925</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>418–419 (Bertarelli 1925, cart. 4, tra pp. 736–737)</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>«Frattocchie» è registrato sulla cart. 4 della Guida 1925 (topografia della guida in QP).</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N120" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>T-0004</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_torraccio</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1925</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>418–419 (Bertarelli 1925, cart. 4, tra pp. 736–737)</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>«Torraccio» è registrato sulla cart. 4 della Guida 1925 (topografia della guida in QP).</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>T-0005</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_due_santi</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1925</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>418–419 (Bertarelli 1925, cart. 4, tra pp. 736–737)</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>«Due Santi» è registrato sulla cart. 4 della Guida 1925 (topografia della guida in QP).</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>T-0006</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_ponte_di_santa_fumia</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1925</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>418–419 (Bertarelli 1925, cart. 4, tra pp. 736–737)</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>«Ponte di Santa Fumia» è registrato sulla cart. 4 della Guida 1925 (topografia della guida in QP).</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>T-0007</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_casale_abbruciato</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1925</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>418–419 (Bertarelli 1925, cart. 4, tra pp. 736–737)</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>«Casal Abbruciato» è registrato sulla cart. 4 della Guida 1925 (topografia della guida in QP).</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>T-0008</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_ponte_divino_amore</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1925</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>418–419 (Bertarelli 1925, cart. 4, tra pp. 736–737)</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>«Ponte del Divino Amore» è registrato sulla cart. 4 della Guida 1925 (topografia della guida in QP).</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>T-0009</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_pavona</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1925</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>418–419 (Bertarelli 1925, cart. 4, tra pp. 736–737)</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>«Pavona» è registrato sulla cart. 4 della Guida 1925 (topografia della guida in QP).</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N126" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>T-0010</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_solforata</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1925</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>418–419 (Bertarelli 1925, cart. 4, tra pp. 736–737)</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>«Zolforata» è registrato sulla cart. 4 della Guida 1925 (topografia della guida in QP).</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>T-0011</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_pratica_di_mare</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1925</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>418–419 (Bertarelli 1925, cart. 4, tra pp. 736–737)</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>«Pratica di Mare» è registrato sulla cart. 4 della Guida 1925 (topografia della guida in QP).</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>T-0012</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_ca_francesi</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1925</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>418–419 (Bertarelli 1925, cart. 4, tra pp. 736–737)</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>«Ca' dei Francesi» è registrato sulla cart. 4 della Guida 1925 (topografia della guida in QP).</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N129" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>T-0013</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_falcognana</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1925</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>418–419 (Bertarelli 1925, cart. 4, tra pp. 736–737)</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>«Falcognana» è registrato sulla cart. 4 della Guida 1925 (topografia della guida in QP).</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>T-0014</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_cecchina</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1925</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>418–419 (Bertarelli 1925, cart. 4, tra pp. 736–737)</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>«Cecchina» è registrato sulla cart. 4 della Guida 1925 (topografia della guida in QP).</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N131" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>T-0015</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_albano_laziale</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1925</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>418–419 (Bertarelli 1925, cart. 4, tra pp. 736–737)</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>«Albano» è registrato sulla cart. 4 della Guida 1925 (topografia della guida in QP).</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N132" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>T-0016</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_zagarolo</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1925</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>418–419 (Bertarelli 1925, cart. 4, tra pp. 736–737)</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>«Zagarolo» è registrato sulla cart. 4 della Guida 1925 (topografia della guida in QP).</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N133" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>T-0017</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_marino</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1925</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>418–419 (Bertarelli 1925, cart. 4, tra pp. 736–737)</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>«Marino» è registrato sulla cart. 4 della Guida 1925 (topografia della guida in QP).</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N134" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>T-0018</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_ariccia</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1925</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>418–419 (Bertarelli 1925, cart. 4, tra pp. 736–737)</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>«Ariccia» è registrato sulla cart. 4 della Guida 1925 (topografia della guida in QP).</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N135" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>T-0019</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_santa_palomba</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1925</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>418–419 (Bertarelli 1925, cart. 4, tra pp. 736–737)</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>«Santa Palomba» è registrato sulla cart. 4 della Guida 1925 (topografia della guida in QP).</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>T-0020</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_rocca_di_papa</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1925</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>418–419 (Bertarelli 1925, cart. 4, tra pp. 736–737)</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>«Rocca di Papa» è registrato sulla cart. 4 della Guida 1925 (topografia della guida in QP).</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>K-0004</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>commentary</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>work/quer_pasticciaccio</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>418–419</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>La topografia di QP è strettamente legata a quella della guida del Touring, anche nelle indicazioni stradali date ai personaggi.</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="T138" t="inlineStr">
+        <is>
+          <t>«la topografia di QP è strettamente legata a quella della guida del Touring»</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>T-0023</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_casale_abbruciato</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1924</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>766 (Bertarelli 1924, cart. 2, tra pp. 480–481)</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>«C. Abbruciato» sulla cartina del 1924; concorde con L-0001.</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="T139" t="inlineStr">
+        <is>
+          <t>«C. Abbruciato»</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>T-0024</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_ponte_di_santa_fumia</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1925</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>911 (Bertarelli 1925, cart. 4, tra pp. 736–737)</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>Ponte di Santa Fumia sulla cart. 4 della Guida 1925.</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>K-0005</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>commentary</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>route/tragitto_torraccio_ponte_divino_amore</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>911 (cfr. Terzoli 2008, pp. 109–113)</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>La strada dall'Anziate a Casal Bruciato, parallela alla Falcognana, corrisponde alla planimetria delle cart. 4 e 1 della Guida 1925.</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="R141" t="inlineStr">
+        <is>
+          <t>ref_00698</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>K-0006</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>commentary</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>narrativeplace/casello_km_20_25</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H142" t="n">
+        <v>911</v>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>Terzoli chiama «immaginario» il casello di Casal Bruciato. Commento attribuito: lo statuto non cambia.</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="T142" t="inlineStr">
+        <is>
+          <t>«immaginario»</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>K-0007</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>commentary</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>narrativeplace/tor_di_gheppio</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H143" t="n">
+        <v>911</v>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>Terzoli chiama «immaginaria» Tor di Gheppio. Commento attribuito: lo statuto non cambia.</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="T143" t="inlineStr">
+        <is>
+          <t>«immaginaria»</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>K-0008</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>commentary</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>route/tragitto_sogno_casal_bruciato_campo_morto</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>manzotti</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>manzotti_2010</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>268–269</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>«Per fil a dest»: passaggio a livello sulla Roma–Velletri presso il casello km 20,25, fra Santa Maria delle Mole (km 17,55) e Pavona (km 23,38); premonizione dell'itinerario di fuga.</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N144" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="R144" t="inlineStr">
+        <is>
+          <t>ref_00534</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>T-0025</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>repertory</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_monti_ernici</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>source/bertarelli_1924</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>696 (Bertarelli 1924, p. 498; cart. 2)</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>I monti Ernici nella Guida 1924, p. 498, e sulla cart. 2.</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N145" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>I-0005</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>identification</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>narrativeplace/tenenza_carabinieri_marino</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_palazzo_colonna_marino</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>manzotti</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>manzotti_2010</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>239–240</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>La caserma è il palazzo Frangipani-Orsini-Colonna su piazza Umberto I (oggi della Repubblica) (TCI, Italia centrale IV, p. 761), non la palazzina in Pierangeli: «re-invenzione romantica». Non adottata: le ancore della tenenza non cambiano.</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="T146" t="inlineStr">
+        <is>
+          <t>«re-invenzione romantica»</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>K-0009</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>commentary</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>narrativeplace/marino</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>manzotti</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>manzotti_2010</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>293–294</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>Marino come topografia familiare (Longone-Lukones) e luogo di delizie enologiche.</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>N-0004</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>naming</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>narrativeplace/castel_porcano</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>chora:Paraetymology</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>manzotti</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>manzotti_2010</t>
+        </is>
+      </c>
+      <c r="H148" t="n">
+        <v>273</v>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Gioco paraetimologico su Castelporziano (Real Tenuta; TCI, Italia centrale I, p. 569); vale anche per «Castel Porcino».</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="R148" t="inlineStr">
+        <is>
+          <t>ref_00538|ref_00539</t>
+        </is>
+      </c>
+      <c r="U148" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_castel_porziano</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>K-0010</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>commentary</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>reference/ref_00539</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>manzotti</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>manzotti_2010</t>
+        </is>
+      </c>
+      <c r="H149" t="n">
+        <v>276</v>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Lo slittamento Porcano → Porcino sottolinea lo spostamento del sogno verso la Zamira.</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="R149" t="inlineStr">
+        <is>
+          <t>ref_00539</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>I-0006</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>identification</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>narrativeplace/palazzo_simonetti</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_palazzo_odescalchi_simonetti</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>535–536</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Palazzo Odescalchi Simonetti, via Vittoria Colonna 11: l'indirizzo romano di Gadda (pensione White).</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="R150" t="inlineStr">
+        <is>
+          <t>ref_00435</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>I-0007</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>identification</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>narrativeplace/palazzo_simonetti</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_palazzo_de_carolis_simonetti</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>grassadonia|lagossi|marchetti</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H151" t="n">
+        <v>536</v>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Palazzo De Carolis Simonetti, via del Corso 307 / via Lata 3.</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>Grassadonia, Lagossi e Marchetti 1997a, cit. in Terzoli 2015, p. 536 (D-087).</t>
+        </is>
+      </c>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="R151" t="inlineStr">
+        <is>
+          <t>ref_00435</t>
+        </is>
+      </c>
+      <c r="S151" t="inlineStr">
+        <is>
+          <t>glm_1997a</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>I-0008</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>identification</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>narrativeplace/palazzo_simonetti</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_palazzo_de_carolis_simonetti</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>pinotti</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>pinotti_2025</t>
+        </is>
+      </c>
+      <c r="H152" t="n">
+        <v>78</v>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Lo stesso edificio, dalla lezione «via Lata» del dattiloscritto dei capitoli nuovi.</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="R152" t="inlineStr">
+        <is>
+          <t>ref_00435|ref_00725</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>N-0005</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>naming</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>reference/ref_00437</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>chora:Synecdoche</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H153" t="n">
+        <v>537</v>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>«Palazzo der Mappamonno»: Palazzo Venezia indicato per sineddoche dalla Sala del Mappamondo.</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="R153" t="inlineStr">
+        <is>
+          <t>ref_00437</t>
+        </is>
+      </c>
+      <c r="U153" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_palazzo_venezia</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>I-0009</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>identification</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>narrativeplace/palazzo_del_mappamondo</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_palazzo_venezia</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H154" t="n">
+        <v>537</v>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Il palazzo der Mappamonno è Palazzo Venezia, sede di Mussolini.</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="R154" t="inlineStr">
+        <is>
+          <t>ref_00437</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>I-0010</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>identification</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>narrativeplace/palazzo_del_mappamondo</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_palazzo_chigi</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>grassadonia|lagossi|marchetti</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H155" t="n">
+        <v>537</v>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Alternativa: Palazzo Chigi (Sala dei Mappamondi).</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>Grassadonia, Lagossi e Marchetti 1997a, cit. in Terzoli 2015, p. 537 (D-087).</t>
+        </is>
+      </c>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="R155" t="inlineStr">
+        <is>
+          <t>ref_00437</t>
+        </is>
+      </c>
+      <c r="S155" t="inlineStr">
+        <is>
+          <t>glm_1997a</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>I-0011</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>identification</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>narrativeplace/vite</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>gazetteer/gaz_via_della_vite</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H156" t="n">
+        <v>616</v>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>«A la Vite» è probabilmente il ristorante Le Grotte, in via della Vite (rione Campo Marzio).</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N156" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="R156" t="inlineStr">
+        <is>
+          <t>ref_00493</t>
+        </is>
+      </c>
+      <c r="T156" t="inlineStr">
+        <is>
+          <t>«probabilmente il ristorante Le Grotte, in via della Vite (nel rione Campo Marzio), uno dei più antichi e rinomati locali romani»</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>V-0006</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>variant</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>reference/ref_00493</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>reference/ref_00735</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>pinotti</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>pinotti_2025</t>
+        </is>
+      </c>
+      <c r="H157" t="n">
+        <v>78</v>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>Il dattiloscritto legge «da Faraja», cioè il Gran Caffè Faraglia, all'angolo fra piazza Venezia e via Cesare Battisti, dove QPa 200 legge «a la Vite».</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N157" t="inlineStr">
+        <is>
+          <t>prova testuale</t>
+        </is>
+      </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+      <c r="R157" t="inlineStr">
+        <is>
+          <t>ref_00493</t>
+        </is>
+      </c>
+      <c r="T157" t="inlineStr">
+        <is>
+          <t>«da Faraja»</t>
+        </is>
+      </c>
+      <c r="V157" t="inlineStr">
+        <is>
+          <t>sostituzione</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>N-0006</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>naming</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>narrativeplace/ditta_ciurlani</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>chora:OnomasticPun</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>terzoli</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>433–435, 644</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>«Ciurlani»: origine onomastica e gioco di parole con «truffaldino».</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>Loci critici (D-087).</t>
+        </is>
+      </c>
+      <c r="N158" t="inlineStr">
+        <is>
+          <t>lettura critica</t>
+        </is>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>validata</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>S-osteriuccia_bivio</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>narrativeplace/osteriuccia_bivio</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>chora:Transformed</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>lorenzo_sabatino</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>terzoli_2015</t>
+        </is>
+      </c>
+      <c r="H159" t="n">
+        <v>776</v>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>Osteria registrata dalla guida del Touring sul bivio fra Appia Antica e strada del Divino Amore, presso le Frattocchie; il testo la rende "osteriuccia" senza nome né collocazione precisa: luogo trasformato, ancorato ai toponimi più prossimi.</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>Motivazione di LS (10/10/2026, D-087).</t>
+        </is>
+      </c>
+      <c r="N159" t="inlineStr">
+        <is>
+          <t>prova referenziale</t>
+        </is>
+      </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>validata</t>
         </is>
       </c>
     </row>

</xml_diff>